<commit_message>
AO ANFA : scénario A = interne (base), scénario B = freelances (repli)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoNCg8NnMhqnD1QgFW3cZV
</commit_message>
<xml_diff>
--- a/ao/anfa-2027/03_BUDGET.xlsx
+++ b/ao/anfa-2027/03_BUDGET.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="189">
   <si>
     <t xml:space="preserve">GRILLE DE COÛTS — AO ANFA 2027, Lot 1 vidéos métiers et formations (Pôle Audiovisuel L'Etudiant)</t>
   </si>
@@ -45,7 +45,7 @@
     <t xml:space="preserve">Source</t>
   </si>
   <si>
-    <t xml:space="preserve">TJM — SCÉNARIO A (freelances, tarifs marché)</t>
+    <t xml:space="preserve">TJM — SCÉNARIO B (repli freelances, tarifs marché — si la bande passante de la cellule est faible)</t>
   </si>
   <si>
     <t xml:space="preserve">Réalisateur·rice-JRI documentaire (réalise et cadre)</t>
@@ -81,7 +81,7 @@
     <t xml:space="preserve">Mixeur·se</t>
   </si>
   <si>
-    <t xml:space="preserve">TAUX — SCÉNARIO B (équipe interne de la cellule vidéo)</t>
+    <t xml:space="preserve">TAUX — SCÉNARIO A (base de l'offre : équipe interne de la cellule vidéo)</t>
   </si>
   <si>
     <t xml:space="preserve">Taux interne (jour/personne, masse salariale)</t>
@@ -99,7 +99,7 @@
     <t xml:space="preserve">COMMUN AUX DEUX SCÉNARIOS</t>
   </si>
   <si>
-    <t xml:space="preserve">Location kit tournage léger (scénario A)</t>
+    <t xml:space="preserve">Location kit tournage léger (scénario B)</t>
   </si>
   <si>
     <t xml:space="preserve">BPU IDFM Grille Coûts Production — reportage / ITW</t>
@@ -267,7 +267,7 @@
     <t xml:space="preserve">FORMAT COURT — vidéo métier ou formation, 60–120 s, verticale, immersive (4 par an minimum)</t>
   </si>
   <si>
-    <t xml:space="preserve">Scénario A = freelances aux tarifs marché · Scénario B = équipe interne de la cellule vidéo (taux 200 €/j). Jours en bleu = modifiables.</t>
+    <t xml:space="preserve">Scénario A (base) = équipe interne de la cellule vidéo (taux 200 €/j) · Scénario B (repli) = freelances aux tarifs marché, si la bande passante est faible. Jours en bleu = modifiables.</t>
   </si>
   <si>
     <t xml:space="preserve">Jours / Qté</t>
@@ -276,13 +276,13 @@
     <t xml:space="preserve">Taux A</t>
   </si>
   <si>
-    <t xml:space="preserve">Coût A (freelances)</t>
+    <t xml:space="preserve">Coût A (interne)</t>
   </si>
   <si>
     <t xml:space="preserve">Taux B</t>
   </si>
   <si>
-    <t xml:space="preserve">Coût B (interne)</t>
+    <t xml:space="preserve">Coût B (freelances)</t>
   </si>
   <si>
     <t xml:space="preserve">PRÉPARATION</t>
@@ -426,21 +426,21 @@
     <t xml:space="preserve">SYNTHÈSE — scénario annuel 2027, comparé au budget maximum du Lot 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Total A (interne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total B (freelances)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COÛT UNITAIRE COMPLET PAR FORMAT (production + part de logistique) — base des prix unitaires pour les bons de commande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format</t>
+  </si>
+  <si>
     <t xml:space="preserve">Coût unitaire A</t>
   </si>
   <si>
-    <t xml:space="preserve">Total A (freelances)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total B (interne)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COÛT UNITAIRE COMPLET PAR FORMAT (production + part de logistique) — base des prix unitaires pour les bons de commande</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format</t>
-  </si>
-  <si>
     <t xml:space="preserve">Coût unitaire B</t>
   </si>
   <si>
@@ -489,16 +489,16 @@
     <t xml:space="preserve">Reste pour la médiatisation après marge plancher</t>
   </si>
   <si>
-    <t xml:space="preserve">ÉCART A → B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Économie de coût de revient si la cellule produit en interne (HT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Écart en % du scénario A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠️ Le coût B est de la masse salariale déjà payée (taux 200 €/j), pas une dépense de trésorerie : il mesure la charge de la cellule, pas un achat. Matériel interne non valorisé (hors référentiel).</t>
+    <t xml:space="preserve">BASCULE A → B (si la cellule n'a pas la bande passante)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surcoût de revient si la production bascule en freelances (HT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surcoût en % du scénario A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⚠️ Le coût A est de la masse salariale déjà payée (taux 200 €/j), pas une dépense de trésorerie : il mesure la charge de la cellule, pas un achat. Matériel interne non valorisé (hors référentiel).</t>
   </si>
   <si>
     <t xml:space="preserve">⚠️ La marge et la répartition médiatisation / marge relèvent des OPS. Le repère ×1,3 n'est affiché que pour visualiser ce qu'il reste à la diffusion ; ce n'est pas une décision.</t>
@@ -1149,7 +1149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1241,7 +1241,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
@@ -1723,20 +1723,20 @@
         <v>0.5</v>
       </c>
       <c r="C7" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <f aca="false">B7*C7</f>
+        <v>100</v>
+      </c>
+      <c r="E7" s="15" t="n">
         <f aca="false">Hypothèses!$B$5</f>
         <v>600</v>
       </c>
-      <c r="D7" s="16" t="n">
-        <f aca="false">B7*C7</f>
-        <v>300</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F7" s="16" t="n">
         <f aca="false">B7*E7</f>
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1747,20 +1747,20 @@
         <v>0.5</v>
       </c>
       <c r="C8" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <f aca="false">B8*C8</f>
+        <v>100</v>
+      </c>
+      <c r="E8" s="15" t="n">
         <f aca="false">Hypothèses!$B$6</f>
         <v>500</v>
       </c>
-      <c r="D8" s="16" t="n">
-        <f aca="false">B8*C8</f>
-        <v>250</v>
-      </c>
-      <c r="E8" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F8" s="16" t="n">
         <f aca="false">B8*E8</f>
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1771,20 +1771,20 @@
         <v>0.5</v>
       </c>
       <c r="C9" s="15" t="n">
+        <f aca="false">Hypothèses!$B$13</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <f aca="false">B9*C9</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="15" t="n">
         <f aca="false">Hypothèses!$B$15</f>
         <v>300</v>
       </c>
-      <c r="D9" s="16" t="n">
-        <f aca="false">B9*C9</f>
-        <v>150</v>
-      </c>
-      <c r="E9" s="15" t="n">
-        <f aca="false">Hypothèses!$B$13</f>
-        <v>0</v>
-      </c>
       <c r="F9" s="16" t="n">
         <f aca="false">B9*E9</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1829,20 +1829,20 @@
         <v>1.5</v>
       </c>
       <c r="C12" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <f aca="false">B12*C12</f>
+        <v>300</v>
+      </c>
+      <c r="E12" s="15" t="n">
         <f aca="false">Hypothèses!$B$7</f>
         <v>500</v>
       </c>
-      <c r="D12" s="16" t="n">
-        <f aca="false">B12*C12</f>
-        <v>750</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F12" s="16" t="n">
         <f aca="false">B12*E12</f>
-        <v>300</v>
+        <v>750</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1853,20 +1853,20 @@
         <v>0.5</v>
       </c>
       <c r="C13" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <f aca="false">B13*C13</f>
+        <v>100</v>
+      </c>
+      <c r="E13" s="15" t="n">
         <f aca="false">Hypothèses!$B$8</f>
         <v>600</v>
       </c>
-      <c r="D13" s="16" t="n">
-        <f aca="false">B13*C13</f>
-        <v>300</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F13" s="16" t="n">
         <f aca="false">B13*E13</f>
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1877,20 +1877,20 @@
         <v>0.25</v>
       </c>
       <c r="C14" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <f aca="false">B14*C14</f>
+        <v>50</v>
+      </c>
+      <c r="E14" s="15" t="n">
         <f aca="false">Hypothèses!$B$9</f>
         <v>480</v>
       </c>
-      <c r="D14" s="16" t="n">
-        <f aca="false">B14*C14</f>
-        <v>120</v>
-      </c>
-      <c r="E14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F14" s="16" t="n">
         <f aca="false">B14*E14</f>
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1901,20 +1901,20 @@
         <v>0.25</v>
       </c>
       <c r="C15" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <f aca="false">B15*C15</f>
+        <v>50</v>
+      </c>
+      <c r="E15" s="15" t="n">
         <f aca="false">Hypothèses!$B$10</f>
         <v>480</v>
       </c>
-      <c r="D15" s="16" t="n">
-        <f aca="false">B15*C15</f>
-        <v>120</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F15" s="16" t="n">
         <f aca="false">B15*E15</f>
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1925,20 +1925,20 @@
         <v>0.25</v>
       </c>
       <c r="C16" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <f aca="false">B16*C16</f>
+        <v>50</v>
+      </c>
+      <c r="E16" s="15" t="n">
         <f aca="false">Hypothèses!$B$7</f>
         <v>500</v>
       </c>
-      <c r="D16" s="16" t="n">
-        <f aca="false">B16*C16</f>
-        <v>125</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F16" s="16" t="n">
         <f aca="false">B16*E16</f>
-        <v>50</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1949,20 +1949,20 @@
         <v>0.5</v>
       </c>
       <c r="C17" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <f aca="false">B17*C17</f>
+        <v>100</v>
+      </c>
+      <c r="E17" s="15" t="n">
         <f aca="false">Hypothèses!$B$7</f>
         <v>500</v>
       </c>
-      <c r="D17" s="16" t="n">
-        <f aca="false">B17*C17</f>
-        <v>250</v>
-      </c>
-      <c r="E17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F17" s="16" t="n">
         <f aca="false">B17*E17</f>
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1997,12 +1997,12 @@
       <c r="C19" s="3"/>
       <c r="D19" s="17" t="n">
         <f aca="false">SUM(D5:D18)</f>
-        <v>2565</v>
+        <v>1050</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="17" t="n">
         <f aca="false">SUM(F5:F18)</f>
-        <v>1050</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">D19*C20</f>
-        <v>384.75</v>
+        <v>157.5</v>
       </c>
       <c r="E20" s="18" t="n">
         <f aca="false">Hypothèses!$B$17</f>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="F20" s="16" t="n">
         <f aca="false">F19*E20</f>
-        <v>157.5</v>
+        <v>384.75</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="D21" s="16" t="n">
         <f aca="false">D19*C21</f>
-        <v>76.95</v>
+        <v>31.5</v>
       </c>
       <c r="E21" s="18" t="n">
         <f aca="false">Hypothèses!$B$18</f>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="F21" s="16" t="n">
         <f aca="false">F19*E21</f>
-        <v>31.5</v>
+        <v>76.95</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="D22" s="16" t="n">
         <f aca="false">D19*C22</f>
-        <v>128.25</v>
+        <v>52.5</v>
       </c>
       <c r="E22" s="18" t="n">
         <f aca="false">Hypothèses!$B$19</f>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="F22" s="16" t="n">
         <f aca="false">F19*E22</f>
-        <v>52.5</v>
+        <v>128.25</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2076,12 +2076,12 @@
       <c r="C23" s="3"/>
       <c r="D23" s="17" t="n">
         <f aca="false">D19+D20+D21+D22</f>
-        <v>3154.95</v>
+        <v>1291.5</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="17" t="n">
         <f aca="false">F19+F20+F21+F22</f>
-        <v>1291.5</v>
+        <v>3154.95</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2183,20 +2183,20 @@
         <v>1.5</v>
       </c>
       <c r="C5" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <f aca="false">B5*C5</f>
+        <v>300</v>
+      </c>
+      <c r="E5" s="15" t="n">
         <f aca="false">Hypothèses!$B$5</f>
         <v>600</v>
       </c>
-      <c r="D5" s="16" t="n">
-        <f aca="false">B5*C5</f>
-        <v>900</v>
-      </c>
-      <c r="E5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F5" s="16" t="n">
         <f aca="false">B5*E5</f>
-        <v>300</v>
+        <v>900</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2241,20 +2241,20 @@
         <v>2</v>
       </c>
       <c r="C8" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <f aca="false">B8*C8</f>
+        <v>400</v>
+      </c>
+      <c r="E8" s="15" t="n">
         <f aca="false">Hypothèses!$B$5</f>
         <v>600</v>
       </c>
-      <c r="D8" s="16" t="n">
-        <f aca="false">B8*C8</f>
-        <v>1200</v>
-      </c>
-      <c r="E8" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F8" s="16" t="n">
         <f aca="false">B8*E8</f>
-        <v>400</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2265,20 +2265,20 @@
         <v>2</v>
       </c>
       <c r="C9" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <f aca="false">B9*C9</f>
+        <v>400</v>
+      </c>
+      <c r="E9" s="15" t="n">
         <f aca="false">Hypothèses!$B$6</f>
         <v>500</v>
       </c>
-      <c r="D9" s="16" t="n">
-        <f aca="false">B9*C9</f>
-        <v>1000</v>
-      </c>
-      <c r="E9" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F9" s="16" t="n">
         <f aca="false">B9*E9</f>
-        <v>400</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2289,20 +2289,20 @@
         <v>2</v>
       </c>
       <c r="C10" s="15" t="n">
+        <f aca="false">Hypothèses!$B$13</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <f aca="false">B10*C10</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="15" t="n">
         <f aca="false">Hypothèses!$B$15</f>
         <v>300</v>
       </c>
-      <c r="D10" s="16" t="n">
-        <f aca="false">B10*C10</f>
-        <v>600</v>
-      </c>
-      <c r="E10" s="15" t="n">
-        <f aca="false">Hypothèses!$B$13</f>
-        <v>0</v>
-      </c>
       <c r="F10" s="16" t="n">
         <f aca="false">B10*E10</f>
-        <v>0</v>
+        <v>600</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2347,20 +2347,20 @@
         <v>1.5</v>
       </c>
       <c r="C13" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <f aca="false">B13*C13</f>
+        <v>300</v>
+      </c>
+      <c r="E13" s="15" t="n">
         <f aca="false">Hypothèses!$B$7</f>
         <v>500</v>
       </c>
-      <c r="D13" s="16" t="n">
-        <f aca="false">B13*C13</f>
-        <v>750</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F13" s="16" t="n">
         <f aca="false">B13*E13</f>
-        <v>300</v>
+        <v>750</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2371,20 +2371,20 @@
         <v>5</v>
       </c>
       <c r="C14" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <f aca="false">B14*C14</f>
+        <v>1000</v>
+      </c>
+      <c r="E14" s="15" t="n">
         <f aca="false">Hypothèses!$B$7</f>
         <v>500</v>
       </c>
-      <c r="D14" s="16" t="n">
-        <f aca="false">B14*C14</f>
-        <v>2500</v>
-      </c>
-      <c r="E14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F14" s="16" t="n">
         <f aca="false">B14*E14</f>
-        <v>1000</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2395,20 +2395,20 @@
         <v>1.5</v>
       </c>
       <c r="C15" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <f aca="false">B15*C15</f>
+        <v>300</v>
+      </c>
+      <c r="E15" s="15" t="n">
         <f aca="false">Hypothèses!$B$8</f>
         <v>600</v>
       </c>
-      <c r="D15" s="16" t="n">
-        <f aca="false">B15*C15</f>
-        <v>900</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F15" s="16" t="n">
         <f aca="false">B15*E15</f>
-        <v>300</v>
+        <v>900</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2419,20 +2419,20 @@
         <v>1</v>
       </c>
       <c r="C16" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <f aca="false">B16*C16</f>
+        <v>200</v>
+      </c>
+      <c r="E16" s="15" t="n">
         <f aca="false">Hypothèses!$B$9</f>
         <v>480</v>
       </c>
-      <c r="D16" s="16" t="n">
-        <f aca="false">B16*C16</f>
-        <v>480</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F16" s="16" t="n">
         <f aca="false">B16*E16</f>
-        <v>200</v>
+        <v>480</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2443,20 +2443,20 @@
         <v>1</v>
       </c>
       <c r="C17" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <f aca="false">B17*C17</f>
+        <v>200</v>
+      </c>
+      <c r="E17" s="15" t="n">
         <f aca="false">Hypothèses!$B$10</f>
         <v>480</v>
       </c>
-      <c r="D17" s="16" t="n">
-        <f aca="false">B17*C17</f>
-        <v>480</v>
-      </c>
-      <c r="E17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F17" s="16" t="n">
         <f aca="false">B17*E17</f>
-        <v>200</v>
+        <v>480</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2467,20 +2467,20 @@
         <v>0.5</v>
       </c>
       <c r="C18" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <f aca="false">B18*C18</f>
+        <v>100</v>
+      </c>
+      <c r="E18" s="15" t="n">
         <f aca="false">Hypothèses!$B$7</f>
         <v>500</v>
       </c>
-      <c r="D18" s="16" t="n">
-        <f aca="false">B18*C18</f>
-        <v>250</v>
-      </c>
-      <c r="E18" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F18" s="16" t="n">
         <f aca="false">B18*E18</f>
-        <v>100</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2491,20 +2491,20 @@
         <v>1</v>
       </c>
       <c r="C19" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D19" s="16" t="n">
+        <f aca="false">B19*C19</f>
+        <v>200</v>
+      </c>
+      <c r="E19" s="15" t="n">
         <f aca="false">Hypothèses!$B$7</f>
         <v>500</v>
       </c>
-      <c r="D19" s="16" t="n">
-        <f aca="false">B19*C19</f>
-        <v>500</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F19" s="16" t="n">
         <f aca="false">B19*E19</f>
-        <v>200</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2525,20 +2525,20 @@
         <v>1.5</v>
       </c>
       <c r="C21" s="15" t="n">
+        <f aca="false">Hypothèses!$B$12</f>
+        <v>200</v>
+      </c>
+      <c r="D21" s="16" t="n">
+        <f aca="false">B21*C21</f>
+        <v>300</v>
+      </c>
+      <c r="E21" s="15" t="n">
         <f aca="false">Hypothèses!$B$7</f>
         <v>500</v>
       </c>
-      <c r="D21" s="16" t="n">
-        <f aca="false">B21*C21</f>
-        <v>750</v>
-      </c>
-      <c r="E21" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
-        <v>200</v>
-      </c>
       <c r="F21" s="16" t="n">
         <f aca="false">B21*E21</f>
-        <v>300</v>
+        <v>750</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2573,12 +2573,12 @@
       <c r="C23" s="3"/>
       <c r="D23" s="17" t="n">
         <f aca="false">SUM(D5:D22)</f>
-        <v>10660</v>
+        <v>4050</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="17" t="n">
         <f aca="false">SUM(F5:F22)</f>
-        <v>4050</v>
+        <v>10660</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="D24" s="16" t="n">
         <f aca="false">D23*C24</f>
-        <v>1599</v>
+        <v>607.5</v>
       </c>
       <c r="E24" s="18" t="n">
         <f aca="false">Hypothèses!$B$17</f>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="F24" s="16" t="n">
         <f aca="false">F23*E24</f>
-        <v>607.5</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="D25" s="16" t="n">
         <f aca="false">D23*C25</f>
-        <v>319.8</v>
+        <v>121.5</v>
       </c>
       <c r="E25" s="18" t="n">
         <f aca="false">Hypothèses!$B$18</f>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="F25" s="16" t="n">
         <f aca="false">F23*E25</f>
-        <v>121.5</v>
+        <v>319.8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="D26" s="16" t="n">
         <f aca="false">D23*C26</f>
-        <v>533</v>
+        <v>202.5</v>
       </c>
       <c r="E26" s="18" t="n">
         <f aca="false">Hypothèses!$B$19</f>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="F26" s="16" t="n">
         <f aca="false">F23*E26</f>
-        <v>202.5</v>
+        <v>533</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2652,12 +2652,12 @@
       <c r="C27" s="3"/>
       <c r="D27" s="17" t="n">
         <f aca="false">D23+D24+D25+D26</f>
-        <v>13111.8</v>
+        <v>4981.5</v>
       </c>
       <c r="E27" s="3"/>
       <c r="F27" s="17" t="n">
         <f aca="false">F23+F24+F25+F26</f>
-        <v>4981.5</v>
+        <v>13111.8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2874,19 +2874,17 @@
       <c r="B2" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>134</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -2895,11 +2893,11 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4" t="s">
@@ -2912,11 +2910,11 @@
       </c>
       <c r="C5" s="16" t="n">
         <f aca="false">'Format court'!$D$23+'Logistique vague'!$D$9*Hypothèses!$B$33</f>
-        <v>3522.45</v>
+        <v>1659</v>
       </c>
       <c r="E5" s="16" t="n">
         <f aca="false">'Format court'!$F$23+'Logistique vague'!$D$9*Hypothèses!$B$33</f>
-        <v>1659</v>
+        <v>3522.45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2925,11 +2923,11 @@
       </c>
       <c r="C6" s="16" t="n">
         <f aca="false">'Format long'!$D$27+'Logistique vague'!$D$9*Hypothèses!$B$34</f>
-        <v>13846.8</v>
+        <v>5716.5</v>
       </c>
       <c r="E6" s="16" t="n">
         <f aca="false">'Format long'!$F$27+'Logistique vague'!$D$9*Hypothèses!$B$34</f>
-        <v>5716.5</v>
+        <v>13846.8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2950,10 +2948,10 @@
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>134</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2966,11 +2964,11 @@
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">B10*'Format court'!$D$23</f>
-        <v>12619.8</v>
+        <v>5166</v>
       </c>
       <c r="E10" s="16" t="n">
         <f aca="false">B10*'Format court'!$F$23</f>
-        <v>5166</v>
+        <v>12619.8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2983,11 +2981,11 @@
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">B11*'Format long'!$D$27</f>
-        <v>26223.6</v>
+        <v>9963</v>
       </c>
       <c r="E11" s="16" t="n">
         <f aca="false">B11*'Format long'!$F$27</f>
-        <v>9963</v>
+        <v>26223.6</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3015,11 +3013,11 @@
       <c r="C13" s="3"/>
       <c r="D13" s="17" t="n">
         <f aca="false">SUM(D10:D12)</f>
-        <v>41783.4</v>
+        <v>18069</v>
       </c>
       <c r="E13" s="17" t="n">
         <f aca="false">SUM(E10:E12)</f>
-        <v>18069</v>
+        <v>41783.4</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3037,11 +3035,11 @@
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">D13*Hypothèses!$B$20</f>
-        <v>8356.68</v>
+        <v>3613.8</v>
       </c>
       <c r="E15" s="16" t="n">
         <f aca="false">E13*Hypothèses!$B$20</f>
-        <v>3613.8</v>
+        <v>8356.68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3050,11 +3048,11 @@
       </c>
       <c r="D16" s="24" t="n">
         <f aca="false">D13+D15</f>
-        <v>50140.08</v>
+        <v>21682.8</v>
       </c>
       <c r="E16" s="24" t="n">
         <f aca="false">E13+E15</f>
-        <v>21682.8</v>
+        <v>50140.08</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3085,11 +3083,11 @@
       </c>
       <c r="D20" s="13" t="n">
         <f aca="false">D13/D19</f>
-        <v>0.720403448275862</v>
+        <v>0.311534482758621</v>
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E13/E19</f>
-        <v>0.311534482758621</v>
+        <v>0.720403448275862</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3098,11 +3096,11 @@
       </c>
       <c r="D21" s="24" t="n">
         <f aca="false">D19-D13</f>
-        <v>16216.6</v>
+        <v>39931</v>
       </c>
       <c r="E21" s="24" t="n">
         <f aca="false">E19-E13</f>
-        <v>39931</v>
+        <v>16216.6</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3111,11 +3109,11 @@
       </c>
       <c r="D22" s="16" t="n">
         <f aca="false">D13*Hypothèses!$B$37</f>
-        <v>54318.42</v>
+        <v>23489.7</v>
       </c>
       <c r="E22" s="16" t="n">
         <f aca="false">E13*Hypothèses!$B$37</f>
-        <v>23489.7</v>
+        <v>54318.42</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3124,11 +3122,11 @@
       </c>
       <c r="D23" s="17" t="n">
         <f aca="false">D19-D22</f>
-        <v>3681.58000000001</v>
+        <v>34510.3</v>
       </c>
       <c r="E23" s="17" t="n">
         <f aca="false">E19-E22</f>
-        <v>34510.3</v>
+        <v>3681.58000000001</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3145,7 +3143,7 @@
         <v>155</v>
       </c>
       <c r="E26" s="16" t="n">
-        <f aca="false">D13-E13</f>
+        <f aca="false">E13-D13</f>
         <v>23714.4</v>
       </c>
     </row>
@@ -3154,8 +3152,8 @@
         <v>156</v>
       </c>
       <c r="E27" s="13" t="n">
-        <f aca="false">IF(D13=0,0,(D13-E13)/D13)</f>
-        <v>0.567555536409196</v>
+        <f aca="false">IF(D13=0,0,(E13-D13)/D13)</f>
+        <v>1.31243566329072</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3276,11 +3274,11 @@
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">2*'Format court'!$D$23+'Format long'!$D$27+'Logistique vague'!$D$9</f>
-        <v>20891.7</v>
+        <v>9034.5</v>
       </c>
       <c r="E5" s="16" t="n">
         <f aca="false">2*'Format court'!$F$23+'Format long'!$F$27+'Logistique vague'!$D$9</f>
-        <v>9034.5</v>
+        <v>20891.7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3317,11 +3315,11 @@
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">2*'Format court'!$D$23+'Format long'!$D$27+'Logistique vague'!$D$9</f>
-        <v>20891.7</v>
+        <v>9034.5</v>
       </c>
       <c r="E8" s="16" t="n">
         <f aca="false">2*'Format court'!$F$23+'Format long'!$F$27+'Logistique vague'!$D$9</f>
-        <v>9034.5</v>
+        <v>20891.7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3365,11 +3363,11 @@
       <c r="C12" s="3"/>
       <c r="D12" s="17" t="n">
         <f aca="false">D5+D8</f>
-        <v>41783.4</v>
+        <v>18069</v>
       </c>
       <c r="E12" s="17" t="n">
         <f aca="false">E5+E8</f>
-        <v>18069</v>
+        <v>41783.4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
AO ANFA : scénario B avec JRI au tarif de la grille (550 €/j) à la place du réalisateur
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoNCg8NnMhqnD1QgFW3cZV
</commit_message>
<xml_diff>
--- a/ao/anfa-2027/03_BUDGET.xlsx
+++ b/ao/anfa-2027/03_BUDGET.xlsx
@@ -48,13 +48,13 @@
     <t xml:space="preserve">TJM — SCÉNARIO B (repli freelances, tarifs marché — si la bande passante de la cellule est faible)</t>
   </si>
   <si>
-    <t xml:space="preserve">Réalisateur·rice-JRI documentaire (réalise et cadre)</t>
+    <t xml:space="preserve">JRI — cadreur/journaliste reporter d'images (réalise et cadre sur le terrain)</t>
   </si>
   <si>
     <t xml:space="preserve">€/j</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimation marché Malt (réal doc/branded, hors pub) — à confirmer ; la grille BPU ne donne que le réal pub (1 200 €/j)</t>
+    <t xml:space="preserve">BPU IDFM Grille Coûts Production — COMETES / Malt (tarif en vigueur de la grille). Remplace le réalisateur (décision Martin, 28/10)</t>
   </si>
   <si>
     <t xml:space="preserve">Ingénieur·e du son / 2e caméra</t>
@@ -147,7 +147,7 @@
     <t xml:space="preserve">pers</t>
   </si>
   <si>
-    <t xml:space="preserve">Équipe légère : réal-JRI + son / 2e caméra (sobriété, critère RSE)</t>
+    <t xml:space="preserve">Équipe légère : JRI + son / 2e caméra (sobriété, critère RSE)</t>
   </si>
   <si>
     <t xml:space="preserve">Jours de tournage par vague</t>
@@ -294,7 +294,7 @@
     <t xml:space="preserve">TOURNAGE (½ journée, mutualisée avec le format long sur le même site)</t>
   </si>
   <si>
-    <t xml:space="preserve">Réalisateur·rice-JRI</t>
+    <t xml:space="preserve">JRI (réalise et cadre)</t>
   </si>
   <si>
     <t xml:space="preserve">Kit tournage léger</t>
@@ -1162,7 +1162,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>8</v>
@@ -1732,11 +1732,11 @@
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">Hypothèses!$B$5</f>
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="F7" s="16" t="n">
         <f aca="false">B7*E7</f>
-        <v>300</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2002,7 +2002,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="17" t="n">
         <f aca="false">SUM(F5:F18)</f>
-        <v>2565</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="F20" s="16" t="n">
         <f aca="false">F19*E20</f>
-        <v>384.75</v>
+        <v>381</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="F21" s="16" t="n">
         <f aca="false">F19*E21</f>
-        <v>76.95</v>
+        <v>76.2</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="F22" s="16" t="n">
         <f aca="false">F19*E22</f>
-        <v>128.25</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2081,7 +2081,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="17" t="n">
         <f aca="false">F19+F20+F21+F22</f>
-        <v>3154.95</v>
+        <v>3124.2</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2192,11 +2192,11 @@
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">Hypothèses!$B$5</f>
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="F5" s="16" t="n">
         <f aca="false">B5*E5</f>
-        <v>900</v>
+        <v>825</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2250,11 +2250,11 @@
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">Hypothèses!$B$5</f>
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="F8" s="16" t="n">
         <f aca="false">B8*E8</f>
-        <v>1200</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2578,7 +2578,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="17" t="n">
         <f aca="false">SUM(F5:F22)</f>
-        <v>10660</v>
+        <v>10485</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="F24" s="16" t="n">
         <f aca="false">F23*E24</f>
-        <v>1599</v>
+        <v>1572.75</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="F25" s="16" t="n">
         <f aca="false">F23*E25</f>
-        <v>319.8</v>
+        <v>314.55</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="F26" s="16" t="n">
         <f aca="false">F23*E26</f>
-        <v>533</v>
+        <v>524.25</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2657,7 +2657,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="17" t="n">
         <f aca="false">F23+F24+F25+F26</f>
-        <v>13111.8</v>
+        <v>12896.55</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="E5" s="16" t="n">
         <f aca="false">'Format court'!$F$23+'Logistique vague'!$D$9*Hypothèses!$B$33</f>
-        <v>3522.45</v>
+        <v>3491.7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="E6" s="16" t="n">
         <f aca="false">'Format long'!$F$27+'Logistique vague'!$D$9*Hypothèses!$B$34</f>
-        <v>13846.8</v>
+        <v>13631.55</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="E10" s="16" t="n">
         <f aca="false">B10*'Format court'!$F$23</f>
-        <v>12619.8</v>
+        <v>12496.8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="E11" s="16" t="n">
         <f aca="false">B11*'Format long'!$F$27</f>
-        <v>26223.6</v>
+        <v>25793.1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3017,7 +3017,7 @@
       </c>
       <c r="E13" s="17" t="n">
         <f aca="false">SUM(E10:E12)</f>
-        <v>41783.4</v>
+        <v>41229.9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="E15" s="16" t="n">
         <f aca="false">E13*Hypothèses!$B$20</f>
-        <v>8356.68</v>
+        <v>8245.98</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="E16" s="24" t="n">
         <f aca="false">E13+E15</f>
-        <v>50140.08</v>
+        <v>49475.88</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E13/E19</f>
-        <v>0.720403448275862</v>
+        <v>0.710860344827586</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="E21" s="24" t="n">
         <f aca="false">E19-E13</f>
-        <v>16216.6</v>
+        <v>16770.1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="E22" s="16" t="n">
         <f aca="false">E13*Hypothèses!$B$37</f>
-        <v>54318.42</v>
+        <v>53598.87</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="E23" s="17" t="n">
         <f aca="false">E19-E22</f>
-        <v>3681.58000000001</v>
+        <v>4401.13000000001</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3144,7 +3144,7 @@
       </c>
       <c r="E26" s="16" t="n">
         <f aca="false">E13-D13</f>
-        <v>23714.4</v>
+        <v>23160.9</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">IF(D13=0,0,(E13-D13)/D13)</f>
-        <v>1.31243566329072</v>
+        <v>1.28180308816205</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="E5" s="16" t="n">
         <f aca="false">2*'Format court'!$F$23+'Format long'!$F$27+'Logistique vague'!$D$9</f>
-        <v>20891.7</v>
+        <v>20614.95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="E8" s="16" t="n">
         <f aca="false">2*'Format court'!$F$23+'Format long'!$F$27+'Logistique vague'!$D$9</f>
-        <v>20891.7</v>
+        <v>20614.95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="E12" s="17" t="n">
         <f aca="false">E5+E8</f>
-        <v>41783.4</v>
+        <v>41229.9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
AO ANFA : scénario B mixte (tournages en freelances, écriture et post-prod en interne)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoNCg8NnMhqnD1QgFW3cZV
</commit_message>
<xml_diff>
--- a/ao/anfa-2027/03_BUDGET.xlsx
+++ b/ao/anfa-2027/03_BUDGET.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="183">
   <si>
     <t xml:space="preserve">GRILLE DE COÛTS — AO ANFA 2027, Lot 1 vidéos métiers et formations (Pôle Audiovisuel L'Etudiant)</t>
   </si>
@@ -45,7 +45,7 @@
     <t xml:space="preserve">Source</t>
   </si>
   <si>
-    <t xml:space="preserve">TJM — SCÉNARIO B (repli freelances, tarifs marché — si la bande passante de la cellule est faible)</t>
+    <t xml:space="preserve">TJM — SCÉNARIO B (repli mixte, si la bande passante est faible : freelances sur les tournages, écriture et post-prod en interne)</t>
   </si>
   <si>
     <t xml:space="preserve">JRI — cadreur/journaliste reporter d'images (réalise et cadre sur le terrain)</t>
@@ -63,24 +63,6 @@
     <t xml:space="preserve">BPU IDFM Grille Coûts Production — COMETES / CCPA</t>
   </si>
   <si>
-    <t xml:space="preserve">Monteur·se</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BPU IDFM Grille Coûts Production — COMETES / Malt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motion designer (habillage Métiers Services Auto)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BPU IDFM Grille Coûts Production — Marché pub / Malt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Étalonneur·se</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mixeur·se</t>
-  </si>
-  <si>
     <t xml:space="preserve">TAUX — SCÉNARIO A (base de l'offre : équipe interne de la cellule vidéo)</t>
   </si>
   <si>
@@ -267,7 +249,7 @@
     <t xml:space="preserve">FORMAT COURT — vidéo métier ou formation, 60–120 s, verticale, immersive (4 par an minimum)</t>
   </si>
   <si>
-    <t xml:space="preserve">Scénario A (base) = équipe interne de la cellule vidéo (taux 200 €/j) · Scénario B (repli) = freelances aux tarifs marché, si la bande passante est faible. Jours en bleu = modifiables.</t>
+    <t xml:space="preserve">Scénario A (base) = tout en interne (taux 200 €/j) · Scénario B (repli mixte) = tournages en freelances (JRI + son, kit loué), écriture et post-prod en interne. Jours en bleu = modifiables.</t>
   </si>
   <si>
     <t xml:space="preserve">Jours / Qté</t>
@@ -282,7 +264,7 @@
     <t xml:space="preserve">Taux B</t>
   </si>
   <si>
-    <t xml:space="preserve">Coût B (freelances)</t>
+    <t xml:space="preserve">Coût B (mixte)</t>
   </si>
   <si>
     <t xml:space="preserve">PRÉPARATION</t>
@@ -429,7 +411,7 @@
     <t xml:space="preserve">Total A (interne)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total B (freelances)</t>
+    <t xml:space="preserve">Total B (mixte)</t>
   </si>
   <si>
     <t xml:space="preserve">COÛT UNITAIRE COMPLET PAR FORMAT (production + part de logistique) — base des prix unitaires pour les bons de commande</t>
@@ -492,7 +474,7 @@
     <t xml:space="preserve">BASCULE A → B (si la cellule n'a pas la bande passante)</t>
   </si>
   <si>
-    <t xml:space="preserve">Surcoût de revient si la production bascule en freelances (HT)</t>
+    <t xml:space="preserve">Surcoût de revient si les tournages basculent en freelances (HT)</t>
   </si>
   <si>
     <t xml:space="preserve">Surcoût en % du scénario A</t>
@@ -1110,7 +1092,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
@@ -1149,7 +1131,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1185,420 +1167,364 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>500</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>13</v>
-      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="6" t="n">
-        <v>480</v>
-      </c>
-      <c r="C10" s="7" t="s">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="D11" s="8" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>0.15</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
+      <c r="A14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="6" t="n">
-        <v>300</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>8</v>
-      </c>
       <c r="D15" s="8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="6" t="n">
-        <v>50</v>
+        <v>29</v>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>0.2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="9" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="8" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="9" t="n">
-        <v>0.03</v>
+      <c r="B18" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" s="9" t="n">
-        <v>0.05</v>
+        <v>35</v>
+      </c>
+      <c r="B19" s="10" t="n">
+        <v>3</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" s="9" t="n">
-        <v>0.2</v>
+        <v>38</v>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>3</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
+      <c r="A21" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>2</v>
+        <v>44</v>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>95</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B23" s="10" t="n">
-        <v>3</v>
+        <v>47</v>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>40</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B24" s="10" t="n">
-        <v>3</v>
+        <v>50</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>70</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>150</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>49</v>
-      </c>
+      <c r="A25" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" s="6" t="n">
-        <v>95</v>
+        <v>53</v>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B27" s="6" t="n">
-        <v>40</v>
+        <v>56</v>
+      </c>
+      <c r="B27" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" s="6" t="n">
-        <v>70</v>
+        <v>59</v>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
+      <c r="A29" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" s="10" t="n">
-        <v>2</v>
+        <v>63</v>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>0.5</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>64</v>
-      </c>
+      <c r="A31" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B32" s="10" t="n">
-        <v>2</v>
+        <v>66</v>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>58000</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B33" s="9" t="n">
-        <v>0.25</v>
+        <v>68</v>
+      </c>
+      <c r="B33" s="11" t="n">
+        <v>1.3</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B34" s="9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
+      <c r="A34" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
+      <c r="B34" s="13" t="n">
+        <f aca="false">2*B29+B30</f>
+        <v>1</v>
+      </c>
+      <c r="D34" s="12" t="s">
         <v>72</v>
-      </c>
-      <c r="B36" s="6" t="n">
-        <v>58000</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B37" s="11" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B38" s="13" t="n">
-        <f aca="false">2*B33+B34</f>
-        <v>1</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1633,7 +1559,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1643,7 +1569,7 @@
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1656,24 +1582,24 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1683,13 +1609,13 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>0.5</v>
       </c>
       <c r="C5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D5" s="16" t="n">
@@ -1697,7 +1623,7 @@
         <v>100</v>
       </c>
       <c r="E5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="F5" s="16" t="n">
@@ -1707,7 +1633,7 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1717,13 +1643,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>0.5</v>
       </c>
       <c r="C7" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D7" s="16" t="n">
@@ -1747,7 +1673,7 @@
         <v>0.5</v>
       </c>
       <c r="C8" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D8" s="16" t="n">
@@ -1765,13 +1691,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>0.5</v>
       </c>
       <c r="C9" s="15" t="n">
-        <f aca="false">Hypothèses!$B$13</f>
+        <f aca="false">Hypothèses!$B$9</f>
         <v>0</v>
       </c>
       <c r="D9" s="16" t="n">
@@ -1779,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="15" t="n">
-        <f aca="false">Hypothèses!$B$15</f>
+        <f aca="false">Hypothèses!$B$11</f>
         <v>300</v>
       </c>
       <c r="F9" s="16" t="n">
@@ -1789,13 +1715,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>0.25</v>
       </c>
       <c r="C10" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D10" s="16" t="n">
@@ -1803,7 +1729,7 @@
         <v>50</v>
       </c>
       <c r="E10" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="F10" s="16" t="n">
@@ -1813,7 +1739,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -1823,13 +1749,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B12" s="14" t="n">
         <v>1.5</v>
       </c>
       <c r="C12" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D12" s="16" t="n">
@@ -1837,23 +1763,23 @@
         <v>300</v>
       </c>
       <c r="E12" s="15" t="n">
-        <f aca="false">Hypothèses!$B$7</f>
-        <v>500</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F12" s="16" t="n">
         <f aca="false">B12*E12</f>
-        <v>750</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B13" s="14" t="n">
         <v>0.5</v>
       </c>
       <c r="C13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D13" s="16" t="n">
@@ -1862,22 +1788,22 @@
       </c>
       <c r="E13" s="15" t="n">
         <f aca="false">Hypothèses!$B$8</f>
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="F13" s="16" t="n">
         <f aca="false">B13*E13</f>
-        <v>300</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B14" s="14" t="n">
         <v>0.25</v>
       </c>
       <c r="C14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D14" s="16" t="n">
@@ -1885,23 +1811,23 @@
         <v>50</v>
       </c>
       <c r="E14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$9</f>
-        <v>480</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F14" s="16" t="n">
         <f aca="false">B14*E14</f>
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B15" s="14" t="n">
         <v>0.25</v>
       </c>
       <c r="C15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D15" s="16" t="n">
@@ -1909,23 +1835,23 @@
         <v>50</v>
       </c>
       <c r="E15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$10</f>
-        <v>480</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F15" s="16" t="n">
         <f aca="false">B15*E15</f>
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B16" s="14" t="n">
         <v>0.25</v>
       </c>
       <c r="C16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D16" s="16" t="n">
@@ -1933,23 +1859,23 @@
         <v>50</v>
       </c>
       <c r="E16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$7</f>
-        <v>500</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F16" s="16" t="n">
         <f aca="false">B16*E16</f>
-        <v>125</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B17" s="14" t="n">
         <v>0.5</v>
       </c>
       <c r="C17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D17" s="16" t="n">
@@ -1957,23 +1883,23 @@
         <v>100</v>
       </c>
       <c r="E17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$7</f>
-        <v>500</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F17" s="16" t="n">
         <f aca="false">B17*E17</f>
-        <v>250</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="15" t="n">
-        <f aca="false">Hypothèses!$B$16</f>
+        <f aca="false">Hypothèses!$B$12</f>
         <v>50</v>
       </c>
       <c r="D18" s="16" t="n">
@@ -1981,7 +1907,7 @@
         <v>50</v>
       </c>
       <c r="E18" s="15" t="n">
-        <f aca="false">Hypothèses!$B$16</f>
+        <f aca="false">Hypothèses!$B$12</f>
         <v>50</v>
       </c>
       <c r="F18" s="16" t="n">
@@ -1991,7 +1917,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -2002,15 +1928,15 @@
       <c r="E19" s="3"/>
       <c r="F19" s="17" t="n">
         <f aca="false">SUM(F5:F18)</f>
-        <v>2540</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C20" s="18" t="n">
-        <f aca="false">Hypothèses!$B$17</f>
+        <f aca="false">Hypothèses!$B$13</f>
         <v>0.15</v>
       </c>
       <c r="D20" s="16" t="n">
@@ -2018,20 +1944,20 @@
         <v>157.5</v>
       </c>
       <c r="E20" s="18" t="n">
-        <f aca="false">Hypothèses!$B$17</f>
+        <f aca="false">Hypothèses!$B$13</f>
         <v>0.15</v>
       </c>
       <c r="F20" s="16" t="n">
         <f aca="false">F19*E20</f>
-        <v>381</v>
+        <v>228.75</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C21" s="18" t="n">
-        <f aca="false">Hypothèses!$B$18</f>
+        <f aca="false">Hypothèses!$B$14</f>
         <v>0.03</v>
       </c>
       <c r="D21" s="16" t="n">
@@ -2039,20 +1965,20 @@
         <v>31.5</v>
       </c>
       <c r="E21" s="18" t="n">
-        <f aca="false">Hypothèses!$B$18</f>
+        <f aca="false">Hypothèses!$B$14</f>
         <v>0.03</v>
       </c>
       <c r="F21" s="16" t="n">
         <f aca="false">F19*E21</f>
-        <v>76.2</v>
+        <v>45.75</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C22" s="18" t="n">
-        <f aca="false">Hypothèses!$B$19</f>
+        <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
       <c r="D22" s="16" t="n">
@@ -2060,17 +1986,17 @@
         <v>52.5</v>
       </c>
       <c r="E22" s="18" t="n">
-        <f aca="false">Hypothèses!$B$19</f>
+        <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
       <c r="F22" s="16" t="n">
         <f aca="false">F19*E22</f>
-        <v>127</v>
+        <v>76.25</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -2081,12 +2007,12 @@
       <c r="E23" s="3"/>
       <c r="F23" s="17" t="n">
         <f aca="false">F19+F20+F21+F22</f>
-        <v>3124.2</v>
+        <v>1875.75</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B25" s="19"/>
       <c r="C25" s="19"/>
@@ -2127,7 +2053,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2137,7 +2063,7 @@
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2150,24 +2076,24 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -2177,13 +2103,13 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>1.5</v>
       </c>
       <c r="C5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D5" s="16" t="n">
@@ -2191,23 +2117,23 @@
         <v>300</v>
       </c>
       <c r="E5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$5</f>
-        <v>550</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F5" s="16" t="n">
         <f aca="false">B5*E5</f>
-        <v>825</v>
+        <v>300</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D6" s="16" t="n">
@@ -2215,7 +2141,7 @@
         <v>200</v>
       </c>
       <c r="E6" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="F6" s="16" t="n">
@@ -2225,7 +2151,7 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -2235,13 +2161,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D8" s="16" t="n">
@@ -2265,7 +2191,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D9" s="16" t="n">
@@ -2283,13 +2209,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="15" t="n">
-        <f aca="false">Hypothèses!$B$13</f>
+        <f aca="false">Hypothèses!$B$9</f>
         <v>0</v>
       </c>
       <c r="D10" s="16" t="n">
@@ -2297,7 +2223,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="15" t="n">
-        <f aca="false">Hypothèses!$B$15</f>
+        <f aca="false">Hypothèses!$B$11</f>
         <v>300</v>
       </c>
       <c r="F10" s="16" t="n">
@@ -2307,13 +2233,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B11" s="14" t="n">
         <v>0.5</v>
       </c>
       <c r="C11" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D11" s="16" t="n">
@@ -2321,7 +2247,7 @@
         <v>100</v>
       </c>
       <c r="E11" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="F11" s="16" t="n">
@@ -2331,7 +2257,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -2341,13 +2267,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B13" s="14" t="n">
         <v>1.5</v>
       </c>
       <c r="C13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D13" s="16" t="n">
@@ -2355,23 +2281,23 @@
         <v>300</v>
       </c>
       <c r="E13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$7</f>
-        <v>500</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F13" s="16" t="n">
         <f aca="false">B13*E13</f>
-        <v>750</v>
+        <v>300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B14" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D14" s="16" t="n">
@@ -2379,23 +2305,23 @@
         <v>1000</v>
       </c>
       <c r="E14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$7</f>
-        <v>500</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F14" s="16" t="n">
         <f aca="false">B14*E14</f>
-        <v>2500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B15" s="14" t="n">
         <v>1.5</v>
       </c>
       <c r="C15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D15" s="16" t="n">
@@ -2404,22 +2330,22 @@
       </c>
       <c r="E15" s="15" t="n">
         <f aca="false">Hypothèses!$B$8</f>
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="F15" s="16" t="n">
         <f aca="false">B15*E15</f>
-        <v>900</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B16" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D16" s="16" t="n">
@@ -2427,23 +2353,23 @@
         <v>200</v>
       </c>
       <c r="E16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$9</f>
-        <v>480</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F16" s="16" t="n">
         <f aca="false">B16*E16</f>
-        <v>480</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B17" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D17" s="16" t="n">
@@ -2451,23 +2377,23 @@
         <v>200</v>
       </c>
       <c r="E17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$10</f>
-        <v>480</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F17" s="16" t="n">
         <f aca="false">B17*E17</f>
-        <v>480</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>0.5</v>
       </c>
       <c r="C18" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D18" s="16" t="n">
@@ -2475,23 +2401,23 @@
         <v>100</v>
       </c>
       <c r="E18" s="15" t="n">
-        <f aca="false">Hypothèses!$B$7</f>
-        <v>500</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F18" s="16" t="n">
         <f aca="false">B18*E18</f>
-        <v>250</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B19" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D19" s="16" t="n">
@@ -2499,17 +2425,17 @@
         <v>200</v>
       </c>
       <c r="E19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$7</f>
-        <v>500</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F19" s="16" t="n">
         <f aca="false">B19*E19</f>
-        <v>500</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2519,13 +2445,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B21" s="14" t="n">
         <v>1.5</v>
       </c>
       <c r="C21" s="15" t="n">
-        <f aca="false">Hypothèses!$B$12</f>
+        <f aca="false">Hypothèses!$B$8</f>
         <v>200</v>
       </c>
       <c r="D21" s="16" t="n">
@@ -2533,23 +2459,23 @@
         <v>300</v>
       </c>
       <c r="E21" s="15" t="n">
-        <f aca="false">Hypothèses!$B$7</f>
-        <v>500</v>
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
       </c>
       <c r="F21" s="16" t="n">
         <f aca="false">B21*E21</f>
-        <v>750</v>
+        <v>300</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B22" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="15" t="n">
-        <f aca="false">Hypothèses!$B$16</f>
+        <f aca="false">Hypothèses!$B$12</f>
         <v>50</v>
       </c>
       <c r="D22" s="16" t="n">
@@ -2557,7 +2483,7 @@
         <v>50</v>
       </c>
       <c r="E22" s="15" t="n">
-        <f aca="false">Hypothèses!$B$16</f>
+        <f aca="false">Hypothèses!$B$12</f>
         <v>50</v>
       </c>
       <c r="F22" s="16" t="n">
@@ -2567,7 +2493,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -2578,15 +2504,15 @@
       <c r="E23" s="3"/>
       <c r="F23" s="17" t="n">
         <f aca="false">SUM(F5:F22)</f>
-        <v>10485</v>
+        <v>5950</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C24" s="18" t="n">
-        <f aca="false">Hypothèses!$B$17</f>
+        <f aca="false">Hypothèses!$B$13</f>
         <v>0.15</v>
       </c>
       <c r="D24" s="16" t="n">
@@ -2594,20 +2520,20 @@
         <v>607.5</v>
       </c>
       <c r="E24" s="18" t="n">
-        <f aca="false">Hypothèses!$B$17</f>
+        <f aca="false">Hypothèses!$B$13</f>
         <v>0.15</v>
       </c>
       <c r="F24" s="16" t="n">
         <f aca="false">F23*E24</f>
-        <v>1572.75</v>
+        <v>892.5</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C25" s="18" t="n">
-        <f aca="false">Hypothèses!$B$18</f>
+        <f aca="false">Hypothèses!$B$14</f>
         <v>0.03</v>
       </c>
       <c r="D25" s="16" t="n">
@@ -2615,20 +2541,20 @@
         <v>121.5</v>
       </c>
       <c r="E25" s="18" t="n">
-        <f aca="false">Hypothèses!$B$18</f>
+        <f aca="false">Hypothèses!$B$14</f>
         <v>0.03</v>
       </c>
       <c r="F25" s="16" t="n">
         <f aca="false">F23*E25</f>
-        <v>314.55</v>
+        <v>178.5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C26" s="18" t="n">
-        <f aca="false">Hypothèses!$B$19</f>
+        <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
       <c r="D26" s="16" t="n">
@@ -2636,17 +2562,17 @@
         <v>202.5</v>
       </c>
       <c r="E26" s="18" t="n">
-        <f aca="false">Hypothèses!$B$19</f>
+        <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
       <c r="F26" s="16" t="n">
         <f aca="false">F23*E26</f>
-        <v>524.25</v>
+        <v>297.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2657,12 +2583,12 @@
       <c r="E27" s="3"/>
       <c r="F27" s="17" t="n">
         <f aca="false">F23+F24+F25+F26</f>
-        <v>12896.55</v>
+        <v>7318.5</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B29" s="19"/>
       <c r="C29" s="19"/>
@@ -2701,7 +2627,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2712,82 +2638,82 @@
         <v>2</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C3" s="21" t="n">
-        <f aca="false">Hypothèses!$B$22</f>
+        <f aca="false">Hypothèses!$B$18</f>
         <v>2</v>
       </c>
       <c r="D3" s="16" t="n">
-        <f aca="false">C3*Hypothèses!$B$25</f>
+        <f aca="false">C3*Hypothèses!$B$21</f>
         <v>300</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C4" s="21" t="n">
-        <f aca="false">Hypothèses!$B$22*Hypothèses!$B$24</f>
+        <f aca="false">Hypothèses!$B$18*Hypothèses!$B$20</f>
         <v>6</v>
       </c>
       <c r="D4" s="16" t="n">
-        <f aca="false">C4*Hypothèses!$B$26</f>
+        <f aca="false">C4*Hypothèses!$B$22</f>
         <v>570</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C5" s="21" t="n">
-        <f aca="false">Hypothèses!$B$22*(Hypothèses!$B$23+1)</f>
+        <f aca="false">Hypothèses!$B$18*(Hypothèses!$B$19+1)</f>
         <v>8</v>
       </c>
       <c r="D5" s="16" t="n">
-        <f aca="false">C5*Hypothèses!$B$27</f>
+        <f aca="false">C5*Hypothèses!$B$23</f>
         <v>320</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C6" s="21" t="n">
-        <f aca="false">Hypothèses!$B$23</f>
+        <f aca="false">Hypothèses!$B$19</f>
         <v>3</v>
       </c>
       <c r="D6" s="16" t="n">
-        <f aca="false">C6*Hypothèses!$B$28</f>
+        <f aca="false">C6*Hypothèses!$B$24</f>
         <v>210</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -2798,10 +2724,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C8" s="18" t="n">
-        <f aca="false">Hypothèses!$B$19</f>
+        <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
       <c r="D8" s="16" t="n">
@@ -2811,7 +2737,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -2822,7 +2748,7 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="19"/>
@@ -2860,7 +2786,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2872,19 +2798,19 @@
         <v>2</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -2893,46 +2819,46 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C5" s="16" t="n">
-        <f aca="false">'Format court'!$D$23+'Logistique vague'!$D$9*Hypothèses!$B$33</f>
+        <f aca="false">'Format court'!$D$23+'Logistique vague'!$D$9*Hypothèses!$B$29</f>
         <v>1659</v>
       </c>
       <c r="E5" s="16" t="n">
-        <f aca="false">'Format court'!$F$23+'Logistique vague'!$D$9*Hypothèses!$B$33</f>
-        <v>3491.7</v>
+        <f aca="false">'Format court'!$F$23+'Logistique vague'!$D$9*Hypothèses!$B$29</f>
+        <v>2243.25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C6" s="16" t="n">
-        <f aca="false">'Format long'!$D$27+'Logistique vague'!$D$9*Hypothèses!$B$34</f>
+        <f aca="false">'Format long'!$D$27+'Logistique vague'!$D$9*Hypothèses!$B$30</f>
         <v>5716.5</v>
       </c>
       <c r="E6" s="16" t="n">
-        <f aca="false">'Format long'!$F$27+'Logistique vague'!$D$9*Hypothèses!$B$34</f>
-        <v>13631.55</v>
+        <f aca="false">'Format long'!$F$27+'Logistique vague'!$D$9*Hypothèses!$B$30</f>
+        <v>8053.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -2944,22 +2870,22 @@
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B10" s="21" t="n">
-        <f aca="false">Hypothèses!$B$31</f>
+        <f aca="false">Hypothèses!$B$27</f>
         <v>4</v>
       </c>
       <c r="D10" s="16" t="n">
@@ -2968,15 +2894,15 @@
       </c>
       <c r="E10" s="16" t="n">
         <f aca="false">B10*'Format court'!$F$23</f>
-        <v>12496.8</v>
+        <v>7503</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B11" s="21" t="n">
-        <f aca="false">Hypothèses!$B$32</f>
+        <f aca="false">Hypothèses!$B$28</f>
         <v>2</v>
       </c>
       <c r="D11" s="16" t="n">
@@ -2985,15 +2911,15 @@
       </c>
       <c r="E11" s="16" t="n">
         <f aca="false">B11*'Format long'!$F$27</f>
-        <v>25793.1</v>
+        <v>14637</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="B12" s="21" t="n">
-        <f aca="false">Hypothèses!$B$30</f>
+        <f aca="false">Hypothèses!$B$26</f>
         <v>2</v>
       </c>
       <c r="D12" s="16" t="n">
@@ -3007,7 +2933,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3017,12 +2943,12 @@
       </c>
       <c r="E13" s="17" t="n">
         <f aca="false">SUM(E10:E12)</f>
-        <v>41229.9</v>
+        <v>25080</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">B10+B11*4</f>
@@ -3031,20 +2957,20 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D15" s="16" t="n">
-        <f aca="false">D13*Hypothèses!$B$20</f>
+        <f aca="false">D13*Hypothèses!$B$16</f>
         <v>3613.8</v>
       </c>
       <c r="E15" s="16" t="n">
-        <f aca="false">E13*Hypothèses!$B$20</f>
-        <v>8245.98</v>
+        <f aca="false">E13*Hypothèses!$B$16</f>
+        <v>5016</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D16" s="24" t="n">
         <f aca="false">D13+D15</f>
@@ -3052,12 +2978,12 @@
       </c>
       <c r="E16" s="24" t="n">
         <f aca="false">E13+E15</f>
-        <v>49475.88</v>
+        <v>30096</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -3066,20 +2992,20 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$36</f>
+        <f aca="false">Hypothèses!$B$32</f>
         <v>58000</v>
       </c>
       <c r="E19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$36</f>
+        <f aca="false">Hypothèses!$B$32</f>
         <v>58000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D20" s="13" t="n">
         <f aca="false">D13/D19</f>
@@ -3087,12 +3013,12 @@
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E13/E19</f>
-        <v>0.710860344827586</v>
+        <v>0.432413793103448</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D21" s="24" t="n">
         <f aca="false">D19-D13</f>
@@ -3100,25 +3026,25 @@
       </c>
       <c r="E21" s="24" t="n">
         <f aca="false">E19-E13</f>
-        <v>16770.1</v>
+        <v>32920</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D22" s="16" t="n">
-        <f aca="false">D13*Hypothèses!$B$37</f>
+        <f aca="false">D13*Hypothèses!$B$33</f>
         <v>23489.7</v>
       </c>
       <c r="E22" s="16" t="n">
-        <f aca="false">E13*Hypothèses!$B$37</f>
-        <v>53598.87</v>
+        <f aca="false">E13*Hypothèses!$B$33</f>
+        <v>32604</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D23" s="17" t="n">
         <f aca="false">D19-D22</f>
@@ -3126,12 +3052,12 @@
       </c>
       <c r="E23" s="17" t="n">
         <f aca="false">E19-E22</f>
-        <v>4401.13000000001</v>
+        <v>25396</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -3140,25 +3066,25 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E26" s="16" t="n">
         <f aca="false">E13-D13</f>
-        <v>23160.9</v>
+        <v>7011</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">IF(D13=0,0,(E13-D13)/D13)</f>
-        <v>1.28180308816205</v>
+        <v>0.38801261829653</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B29" s="19"/>
       <c r="C29" s="19"/>
@@ -3167,7 +3093,7 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
@@ -3176,7 +3102,7 @@
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
@@ -3216,7 +3142,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3225,52 +3151,52 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">2*'Format court'!$D$23+'Format long'!$D$27+'Logistique vague'!$D$9</f>
@@ -3278,40 +3204,40 @@
       </c>
       <c r="E5" s="16" t="n">
         <f aca="false">2*'Format court'!$F$23+'Format long'!$F$27+'Logistique vague'!$D$9</f>
-        <v>20614.95</v>
+        <v>12540</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">2*'Format court'!$D$23+'Format long'!$D$27+'Logistique vague'!$D$9</f>
@@ -3319,45 +3245,45 @@
       </c>
       <c r="E8" s="16" t="n">
         <f aca="false">2*'Format court'!$F$23+'Format long'!$F$27+'Logistique vague'!$D$9</f>
-        <v>20614.95</v>
+        <v>12540</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -3367,12 +3293,12 @@
       </c>
       <c r="E12" s="17" t="n">
         <f aca="false">E5+E8</f>
-        <v>41229.9</v>
+        <v>25080</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">D12-Synthèse!$D$13</f>

</xml_diff>

<commit_message>
AO ANFA : logistique intégrée à chaque vidéo (fin de la logique de vagues)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoNCg8NnMhqnD1QgFW3cZV
</commit_message>
<xml_diff>
--- a/ao/anfa-2027/03_BUDGET.xlsx
+++ b/ao/anfa-2027/03_BUDGET.xlsx
@@ -11,9 +11,8 @@
     <sheet name="Hypothèses" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Format court" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Format long" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Logistique vague" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Synthèse" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Calendrier 2027" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Synthèse" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Calendrier 2027" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="172">
   <si>
     <t xml:space="preserve">GRILLE DE COÛTS — AO ANFA 2027, Lot 1 vidéos métiers et formations (Pôle Audiovisuel L'Etudiant)</t>
   </si>
@@ -120,7 +119,7 @@
     <t xml:space="preserve">Taux standard</t>
   </si>
   <si>
-    <t xml:space="preserve">LOGISTIQUE D'UNE VAGUE DE TOURNAGE EN RÉGION</t>
+    <t xml:space="preserve">LOGISTIQUE — TARIFS (déplacement Paris → région, identiques dans les deux scénarios)</t>
   </si>
   <si>
     <t xml:space="preserve">Personnes en déplacement</t>
@@ -132,67 +131,85 @@
     <t xml:space="preserve">Équipe légère : JRI + son / 2e caméra (sobriété, critère RSE)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jours de tournage par vague</t>
+    <t xml:space="preserve">Transport A/R Paris–région par personne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/pers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimation marché — train 2de classe, destination non arrêtée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuitée hôtel par personne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/nuit/pers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimation marché — hôtel pro province (référence CYRCE/BIOT2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per diem repas par personne et par jour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/j/pers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barème URSSAF frais professionnels 2026 — base 2 repas/jour (référence CYRCE/BIOT2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Location véhicule sur place</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimation marché — utilitaire léger / citadine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOGISTIQUE — PAR FORMAT (chaque vidéo est chiffrée seule, déplacement compris)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format court : nuits sur place</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nuits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrivée la veille, 1 journée de tournage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format court : jours de per diem</t>
   </si>
   <si>
     <t xml:space="preserve">j</t>
   </si>
   <si>
-    <t xml:space="preserve">Fiche Approche : J1 entreprise (court métier + long), J2 CFA (court formation + long), J3 long</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nuits sur place par vague</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nuits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arrivée la veille de J1 ; sites potentiellement dans deux villes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transport A/R Paris–région par personne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€/pers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimation marché — train 2de classe, destination non arrêtée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nuitée hôtel par personne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€/nuit/pers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimation marché — hôtel pro province (référence CYRCE/BIOT2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per diem repas par personne et par jour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€/j/pers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barème URSSAF frais professionnels 2026 — base 2 repas/jour (référence CYRCE/BIOT2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Location véhicule sur place</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimation marché — utilitaire léger / citadine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VOLUMES ET CLÉS DE RÉPARTITION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nombre de vagues de tournage par an</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vagues</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calendrier 2027 : fin février–mars, puis mai</t>
+    <t xml:space="preserve">Veille + jour de tournage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format court : jours de véhicule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 journée de tournage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format long : nuits sur place</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrivée la veille, 2 journées de tournage (1 ou 2 sites)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format long : jours de per diem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Veille + 2 jours de tournage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format long : jours de véhicule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 journées de tournage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VOLUMES</t>
   </si>
   <si>
     <t xml:space="preserve">Formats courts par an (60–120 s)</t>
@@ -210,18 +227,6 @@
     <t xml:space="preserve">CDC §3.1 + réponse ANFA du 28/10 : 2 thématiques par an</t>
   </si>
   <si>
-    <t xml:space="preserve">Part de la logistique d'une vague imputée à chaque court</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clé interne : une vague = 2 courts (25 % chacun) + 1 long (50 %)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Part de la logistique d'une vague imputée au long</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clé interne — la somme des clés doit faire 100 %</t>
-  </si>
-  <si>
     <t xml:space="preserve">CADRE CLIENT</t>
   </si>
   <si>
@@ -240,16 +245,10 @@
     <t xml:space="preserve">BPU IDFM — Repères de marge (×1,3 plancher, ×1,5 standard secteur public). Décision OPS</t>
   </si>
   <si>
-    <t xml:space="preserve">Contrôle : somme des clés de répartition d'une vague</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doit afficher 100 %</t>
-  </si>
-  <si>
     <t xml:space="preserve">FORMAT COURT — vidéo métier ou formation, 60–120 s, verticale, immersive (4 par an minimum)</t>
   </si>
   <si>
-    <t xml:space="preserve">Scénario A (base) = tout en interne (taux 200 €/j) · Scénario B (repli mixte) = tournages en freelances (JRI + son, kit loué), écriture et post-prod en interne. Jours en bleu = modifiables.</t>
+    <t xml:space="preserve">Scénario A (base) = tout en interne (taux 200 €/j) · Scénario B (repli mixte) = tournages en freelances (JRI + son, kit loué), écriture et post-prod en interne. Jours en bleu = modifiables. Chaque vidéo est chiffrée seule, déplacement compris.</t>
   </si>
   <si>
     <t xml:space="preserve">Jours / Qté</t>
@@ -273,7 +272,7 @@
     <t xml:space="preserve">Préparation : brief des intervenants, autorisations droit à l'image (mineurs), feuille de route</t>
   </si>
   <si>
-    <t xml:space="preserve">TOURNAGE (½ journée, mutualisée avec le format long sur le même site)</t>
+    <t xml:space="preserve">TOURNAGE (1 journée sur site)</t>
   </si>
   <si>
     <t xml:space="preserve">JRI (réalise et cadre)</t>
@@ -318,10 +317,34 @@
     <t xml:space="preserve">Provision imprévus</t>
   </si>
   <si>
-    <t xml:space="preserve">COÛT DE REVIENT PRODUCTION (HT) — par vidéo, hors logistique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un court est tourné en une demi-journée, sur le même site et le même jour qu'une partie du format long. La logistique (transport, hôtel, repas) est chiffrée dans l'onglet « Logistique vague » et imputée dans la Synthèse.</t>
+    <t xml:space="preserve">Coût de revient production (HT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOGISTIQUE (déplacement en région)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transport A/R Paris–région (par personne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hôtel (personnes × nuits)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per diem repas (personnes × jours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Location véhicule sur place (jours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provision imprévus (logistique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coût logistique (HT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COÛT DE REVIENT COMPLET PAR VIDÉO (HT) — prix unitaire de bon de commande avant marge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chaque court est chiffré comme une commande autonome : 1 journée de tournage, déplacement et nuit sur place compris. Si deux vidéos sont commandées sur un même site, la logistique de l'une disparaît (le CDC autorise plusieurs vidéos par journée de tournage) : économie à répercuter ou non par les OPS.</t>
   </si>
   <si>
     <t xml:space="preserve">FORMAT LONG — vidéo thématique, 10–15 min, verticale, immersive, chapitrée (2 par an minimum)</t>
@@ -336,7 +359,7 @@
     <t xml:space="preserve">Préparation : repérages à distance, brief, autorisations droit à l'image</t>
   </si>
   <si>
-    <t xml:space="preserve">TOURNAGE (2 jours : ½ j sur chaque site des courts + 1 j dédié)</t>
+    <t xml:space="preserve">TOURNAGE (2 journées, sur 1 ou 2 sites)</t>
   </si>
   <si>
     <t xml:space="preserve">Supervision interne</t>
@@ -360,91 +383,52 @@
     <t xml:space="preserve">Déclinaisons courtes (3 extraits de 60 s, ½ j chacune)</t>
   </si>
   <si>
-    <t xml:space="preserve">Les 3 déclinaisons courtes tirées de chaque long répondent à l'appel aux « formats innovants » du CDC et nourrissent la diffusion (6 courts de plus par an pour un coût marginal). Ligne à passer à 0 si les OPS ne la retiennent pas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOGISTIQUE D'UNE VAGUE DE TOURNAGE EN RÉGION (2 courts + 1 long) — identique dans les deux scénarios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calcul</t>
+    <t xml:space="preserve">Chaque long est chiffré comme une commande autonome, déplacement compris. Les 3 déclinaisons courtes répondent à l'appel aux « formats innovants » du CDC (6 courts de plus par an pour un coût marginal) : ligne à passer à 0 si les OPS ne la retiennent pas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SYNTHÈSE — scénario annuel 2027, comparé au budget maximum du Lot 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COÛT UNITAIRE COMPLET PAR VIDÉO (production + logistique) — base des prix unitaires des bons de commande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coût unitaire A (interne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coût unitaire B (mixte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format court (60–120 s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format long (10–15 min) + 3 déclinaisons courtes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCÉNARIO ANNUEL MINIMUM (volumes du cahier des charges)</t>
   </si>
   <si>
     <t xml:space="preserve">Quantité</t>
   </si>
   <si>
-    <t xml:space="preserve">Coût</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transport A/R Paris–région</t>
-  </si>
-  <si>
-    <t xml:space="preserve">personnes × A/R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hôtel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">personnes × nuits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per diem repas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">personnes × (jours de tournage + 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jours de tournage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sous-total logistique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COÛT LOGISTIQUE PAR VAGUE (HT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un seul déplacement sert trois vidéos : c'est l'argument RSE (moins de trajets, empreinte carbone réduite) et la condition pour tenir le budget. Tournages mutualisés acceptés par l'ANFA (réponse du 28/10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SYNTHÈSE — scénario annuel 2027, comparé au budget maximum du Lot 1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total A (interne)</t>
   </si>
   <si>
     <t xml:space="preserve">Total B (mixte)</t>
   </si>
   <si>
-    <t xml:space="preserve">COÛT UNITAIRE COMPLET PAR FORMAT (production + part de logistique) — base des prix unitaires pour les bons de commande</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coût unitaire A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coût unitaire B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format court (60–120 s)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format long (10–15 min) + 3 déclinaisons courtes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCÉNARIO ANNUEL MINIMUM (volumes du cahier des charges)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formats courts — production</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formats longs (avec 3 déclinaisons chacun) — production</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logistique des vagues de tournage en région</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COÛT DE REVIENT PRODUCTION ANNUEL (HT)</t>
+    <t xml:space="preserve">Formats courts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formats longs (avec 3 déclinaisons chacun)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COÛT DE REVIENT PRODUCTION ANNUEL (HT), logistique comprise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   dont logistique (déplacements)</t>
   </si>
   <si>
     <t xml:space="preserve">   Vidéos livrées par an (courts + longs + 3 déclinaisons par long)</t>
@@ -480,6 +464,9 @@
     <t xml:space="preserve">Surcoût en % du scénario A</t>
   </si>
   <si>
+    <t xml:space="preserve">⚠️ Chiffrage prudent : chaque vidéo porte son propre déplacement. Si plusieurs commandes sont tournées sur un même site (autorisé par l'ANFA), la logistique partagée baisse le coût réel : marge de manœuvre pour les OPS.</t>
+  </si>
+  <si>
     <t xml:space="preserve">⚠️ Le coût A est de la masse salariale déjà payée (taux 200 €/j), pas une dépense de trésorerie : il mesure la charge de la cellule, pas un achat. Matériel interne non valorisé (hors référentiel).</t>
   </si>
   <si>
@@ -489,7 +476,7 @@
     <t xml:space="preserve">⚠️ Achats médias : la publicité ciblée vers les mineurs est très restreinte sur les grandes plateformes européennes ; la diffusion organique sur nos canaux reste l'atout principal (à chiffrer par les RS).</t>
   </si>
   <si>
-    <t xml:space="preserve">CALENDRIER 2027 — hypothèse de production en deux vagues (sous réserve de notification en janvier)</t>
+    <t xml:space="preserve">CALENDRIER 2027 — repères indicatifs (accord-cadre à bons de commande, sous réserve d'une notification en janvier)</t>
   </si>
   <si>
     <t xml:space="preserve">Période</t>
@@ -498,82 +485,61 @@
     <t xml:space="preserve">Étape</t>
   </si>
   <si>
-    <t xml:space="preserve">Vidéos concernées</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coût de revient A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coût de revient B</t>
+    <t xml:space="preserve">Commentaire</t>
   </si>
   <si>
     <t xml:space="preserve">Janvier</t>
   </si>
   <si>
-    <t xml:space="preserve">Réunion de lancement ANFA : calage campagnes, sujets, circuit de validation, indicateurs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Février</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préprod vague 1 : choix des sites avec l'ANFA, brief intervenants, autorisations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fin février – mars</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tournage vague 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 court métier + 1 court formation + long n°1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mars – avril</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Post-prod vague 1, validations ANFA, diffusion des courts (choix d'orientation de fin de 3e, portes ouvertes CFA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avril – mai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préprod vague 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tournage vague 2 (avant la période du Bac)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 court métier + 1 court formation + long n°2</t>
+    <t xml:space="preserve">Réunion de lancement ANFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calage sur les campagnes ANFA, choix des sujets de l'année, circuit de validation, indicateurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Février – mai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fenêtre de tournage prioritaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diffusion au moment des choix d'orientation de fin de 3e et des portes ouvertes des CFA ; tournages en CFA pendant les périodes de cours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Par commande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préprod → tournage → post-prod → V1 → V2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environ 3 à 4 semaines par court, 6 à 8 semaines par long, validations ANFA comprises</t>
   </si>
   <si>
     <t xml:space="preserve">Juin – juillet</t>
   </si>
   <si>
-    <t xml:space="preserve">Post-prod vague 2</t>
+    <t xml:space="preserve">Fin des post-prods du premier semestre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rythme ralenti avant l'été</t>
   </si>
   <si>
     <t xml:space="preserve">Septembre – octobre</t>
   </si>
   <si>
-    <t xml:space="preserve">Diffusion de rentrée, déclinaisons, relais prescripteurs</t>
+    <t xml:space="preserve">Seconde fenêtre de tournage et diffusion de rentrée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relais auprès des prescripteurs</t>
   </si>
   <si>
     <t xml:space="preserve">Novembre – décembre</t>
   </si>
   <si>
-    <t xml:space="preserve">Bilan annuel quantitatif et qualitatif (base de la décision de reconduction)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL (doit égaler la Synthèse)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contrôle : écart avec la Synthèse</t>
+    <t xml:space="preserve">Bilan annuel quantitatif et qualitatif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base de la décision de reconduction</t>
   </si>
 </sst>
 </file>
@@ -658,16 +624,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="8"/>
-      <color rgb="FF888888"/>
+      <sz val="9"/>
+      <color rgb="FF008000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF008000"/>
+      <i val="true"/>
+      <sz val="8"/>
+      <color rgb="FF888888"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -739,7 +705,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -788,19 +754,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="169" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -812,19 +770,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -837,6 +807,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1092,7 +1066,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
@@ -1295,7 +1269,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -1321,8 +1295,8 @@
       <c r="A19" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="10" t="n">
-        <v>3</v>
+      <c r="B19" s="6" t="n">
+        <v>150</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>36</v>
@@ -1335,8 +1309,8 @@
       <c r="A20" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="10" t="n">
-        <v>3</v>
+      <c r="B20" s="6" t="n">
+        <v>95</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>39</v>
@@ -1350,7 +1324,7 @@
         <v>41</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>42</v>
@@ -1364,166 +1338,176 @@
         <v>44</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="C22" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="8" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>49</v>
-      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="6" t="n">
-        <v>70</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="8" t="s">
+      <c r="B25" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="D25" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
         <v>53</v>
       </c>
       <c r="B26" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>54</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="B27" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B28" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="9" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
+      <c r="B31" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D30" s="8" t="s">
+      <c r="D31" s="8" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="6" t="n">
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="6" t="n">
         <v>58000</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C34" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D32" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B33" s="11" t="n">
+      <c r="D34" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B35" s="11" t="n">
         <v>1.3</v>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12" t="s">
+      <c r="C35" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B34" s="13" t="n">
-        <f aca="false">2*B29+B30</f>
-        <v>1</v>
-      </c>
-      <c r="D34" s="12" t="s">
+      <c r="D35" s="8" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1546,7 +1530,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -1567,7 +1551,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>74</v>
       </c>
@@ -1611,27 +1595,27 @@
       <c r="A5" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B5" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="C5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D5" s="16" t="n">
+      <c r="C5" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D5" s="14" t="n">
         <f aca="false">B5*C5</f>
         <v>100</v>
       </c>
-      <c r="E5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F5" s="16" t="n">
+      <c r="E5" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F5" s="14" t="n">
         <f aca="false">B5*E5</f>
         <v>100</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>82</v>
       </c>
@@ -1645,94 +1629,94 @@
       <c r="A7" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B7" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C7" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D7" s="16" t="n">
+      <c r="B7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D7" s="14" t="n">
         <f aca="false">B7*C7</f>
-        <v>100</v>
-      </c>
-      <c r="E7" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="E7" s="13" t="n">
         <f aca="false">Hypothèses!$B$5</f>
         <v>550</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="14" t="n">
         <f aca="false">B7*E7</f>
-        <v>275</v>
+        <v>550</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C8" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D8" s="16" t="n">
+      <c r="B8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D8" s="14" t="n">
         <f aca="false">B8*C8</f>
-        <v>100</v>
-      </c>
-      <c r="E8" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="E8" s="13" t="n">
         <f aca="false">Hypothèses!$B$6</f>
         <v>500</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="14" t="n">
         <f aca="false">B8*E8</f>
-        <v>250</v>
+        <v>500</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C9" s="15" t="n">
+      <c r="B9" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="13" t="n">
         <f aca="false">Hypothèses!$B$9</f>
         <v>0</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="14" t="n">
         <f aca="false">B9*C9</f>
         <v>0</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="13" t="n">
         <f aca="false">Hypothèses!$B$11</f>
         <v>300</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="14" t="n">
         <f aca="false">B9*E9</f>
-        <v>150</v>
+        <v>300</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="C10" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D10" s="16" t="n">
+      <c r="C10" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D10" s="14" t="n">
         <f aca="false">B10*C10</f>
         <v>50</v>
       </c>
-      <c r="E10" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F10" s="16" t="n">
+      <c r="E10" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F10" s="14" t="n">
         <f aca="false">B10*E10</f>
         <v>50</v>
       </c>
@@ -1751,22 +1735,22 @@
       <c r="A12" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B12" s="14" t="n">
+      <c r="B12" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="C12" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D12" s="16" t="n">
+      <c r="C12" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D12" s="14" t="n">
         <f aca="false">B12*C12</f>
         <v>300</v>
       </c>
-      <c r="E12" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F12" s="16" t="n">
+      <c r="E12" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F12" s="14" t="n">
         <f aca="false">B12*E12</f>
         <v>300</v>
       </c>
@@ -1775,22 +1759,22 @@
       <c r="A13" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B13" s="14" t="n">
+      <c r="B13" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="C13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D13" s="16" t="n">
+      <c r="C13" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D13" s="14" t="n">
         <f aca="false">B13*C13</f>
         <v>100</v>
       </c>
-      <c r="E13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F13" s="16" t="n">
+      <c r="E13" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F13" s="14" t="n">
         <f aca="false">B13*E13</f>
         <v>100</v>
       </c>
@@ -1799,22 +1783,22 @@
       <c r="A14" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="C14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D14" s="16" t="n">
+      <c r="C14" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D14" s="14" t="n">
         <f aca="false">B14*C14</f>
         <v>50</v>
       </c>
-      <c r="E14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F14" s="16" t="n">
+      <c r="E14" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F14" s="14" t="n">
         <f aca="false">B14*E14</f>
         <v>50</v>
       </c>
@@ -1823,22 +1807,22 @@
       <c r="A15" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="C15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D15" s="16" t="n">
+      <c r="C15" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D15" s="14" t="n">
         <f aca="false">B15*C15</f>
         <v>50</v>
       </c>
-      <c r="E15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F15" s="16" t="n">
+      <c r="E15" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F15" s="14" t="n">
         <f aca="false">B15*E15</f>
         <v>50</v>
       </c>
@@ -1847,22 +1831,22 @@
       <c r="A16" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B16" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="C16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D16" s="16" t="n">
+      <c r="C16" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D16" s="14" t="n">
         <f aca="false">B16*C16</f>
         <v>50</v>
       </c>
-      <c r="E16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F16" s="16" t="n">
+      <c r="E16" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F16" s="14" t="n">
         <f aca="false">B16*E16</f>
         <v>50</v>
       </c>
@@ -1871,22 +1855,22 @@
       <c r="A17" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B17" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="C17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D17" s="16" t="n">
+      <c r="C17" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D17" s="14" t="n">
         <f aca="false">B17*C17</f>
         <v>100</v>
       </c>
-      <c r="E17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F17" s="16" t="n">
+      <c r="E17" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F17" s="14" t="n">
         <f aca="false">B17*E17</f>
         <v>100</v>
       </c>
@@ -1895,22 +1879,22 @@
       <c r="A18" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B18" s="14" t="n">
+      <c r="B18" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="15" t="n">
+      <c r="C18" s="13" t="n">
         <f aca="false">Hypothèses!$B$12</f>
         <v>50</v>
       </c>
-      <c r="D18" s="16" t="n">
+      <c r="D18" s="14" t="n">
         <f aca="false">B18*C18</f>
         <v>50</v>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="E18" s="13" t="n">
         <f aca="false">Hypothèses!$B$12</f>
         <v>50</v>
       </c>
-      <c r="F18" s="16" t="n">
+      <c r="F18" s="14" t="n">
         <f aca="false">B18*E18</f>
         <v>50</v>
       </c>
@@ -1921,109 +1905,272 @@
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
-      <c r="D19" s="17" t="n">
+      <c r="D19" s="15" t="n">
         <f aca="false">SUM(D5:D18)</f>
-        <v>1050</v>
+        <v>1250</v>
       </c>
       <c r="E19" s="3"/>
-      <c r="F19" s="17" t="n">
+      <c r="F19" s="15" t="n">
         <f aca="false">SUM(F5:F18)</f>
-        <v>1525</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="16" t="n">
         <f aca="false">Hypothèses!$B$13</f>
         <v>0.15</v>
       </c>
-      <c r="D20" s="16" t="n">
+      <c r="D20" s="14" t="n">
         <f aca="false">D19*C20</f>
-        <v>157.5</v>
-      </c>
-      <c r="E20" s="18" t="n">
+        <v>187.5</v>
+      </c>
+      <c r="E20" s="16" t="n">
         <f aca="false">Hypothèses!$B$13</f>
         <v>0.15</v>
       </c>
-      <c r="F20" s="16" t="n">
+      <c r="F20" s="14" t="n">
         <f aca="false">F19*E20</f>
-        <v>228.75</v>
+        <v>330</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="18" t="n">
+      <c r="C21" s="16" t="n">
         <f aca="false">Hypothèses!$B$14</f>
         <v>0.03</v>
       </c>
-      <c r="D21" s="16" t="n">
+      <c r="D21" s="14" t="n">
         <f aca="false">D19*C21</f>
-        <v>31.5</v>
-      </c>
-      <c r="E21" s="18" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E21" s="16" t="n">
         <f aca="false">Hypothèses!$B$14</f>
         <v>0.03</v>
       </c>
-      <c r="F21" s="16" t="n">
+      <c r="F21" s="14" t="n">
         <f aca="false">F19*E21</f>
-        <v>45.75</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C22" s="18" t="n">
+      <c r="C22" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
-      <c r="D22" s="16" t="n">
+      <c r="D22" s="14" t="n">
         <f aca="false">D19*C22</f>
-        <v>52.5</v>
-      </c>
-      <c r="E22" s="18" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="E22" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
-      <c r="F22" s="16" t="n">
+      <c r="F22" s="14" t="n">
         <f aca="false">F19*E22</f>
-        <v>76.25</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
-      <c r="D23" s="17" t="n">
+      <c r="D23" s="15" t="n">
         <f aca="false">D19+D20+D21+D22</f>
-        <v>1291.5</v>
+        <v>1537.5</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="17" t="n">
+      <c r="F23" s="15" t="n">
         <f aca="false">F19+F20+F21+F22</f>
-        <v>1875.75</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="17" t="n">
+        <f aca="false">Hypothèses!$B$18</f>
+        <v>2</v>
+      </c>
+      <c r="C25" s="13" t="n">
+        <f aca="false">Hypothèses!$B$19</f>
+        <v>150</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <f aca="false">B25*C25</f>
+        <v>300</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <f aca="false">Hypothèses!$B$19</f>
+        <v>150</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <f aca="false">B25*E25</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B26" s="17" t="n">
+        <f aca="false">Hypothèses!$B$18*Hypothèses!$B$24</f>
+        <v>2</v>
+      </c>
+      <c r="C26" s="13" t="n">
+        <f aca="false">Hypothèses!$B$20</f>
+        <v>95</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <f aca="false">B26*C26</f>
+        <v>190</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <f aca="false">Hypothèses!$B$20</f>
+        <v>95</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <f aca="false">B26*E26</f>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" s="17" t="n">
+        <f aca="false">Hypothèses!$B$18*Hypothèses!$B$25</f>
+        <v>4</v>
+      </c>
+      <c r="C27" s="13" t="n">
+        <f aca="false">Hypothèses!$B$21</f>
+        <v>40</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <f aca="false">B27*C27</f>
+        <v>160</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <f aca="false">Hypothèses!$B$21</f>
+        <v>40</v>
+      </c>
+      <c r="F27" s="14" t="n">
+        <f aca="false">B27*E27</f>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" s="17" t="n">
+        <f aca="false">Hypothèses!$B$26</f>
+        <v>1</v>
+      </c>
+      <c r="C28" s="13" t="n">
+        <f aca="false">Hypothèses!$B$22</f>
+        <v>70</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <f aca="false">B28*C28</f>
+        <v>70</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <f aca="false">Hypothèses!$B$22</f>
+        <v>70</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <f aca="false">B28*E28</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" s="16" t="n">
+        <f aca="false">Hypothèses!$B$15</f>
+        <v>0.05</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <f aca="false">SUM(D25:D28)*C29</f>
+        <v>36</v>
+      </c>
+      <c r="E29" s="16" t="n">
+        <f aca="false">Hypothèses!$B$15</f>
+        <v>0.05</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <f aca="false">SUM(F25:F28)*E29</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="15" t="n">
+        <f aca="false">SUM(D25:D29)</f>
+        <v>756</v>
+      </c>
+      <c r="E30" s="3"/>
+      <c r="F30" s="15" t="n">
+        <f aca="false">SUM(F25:F29)</f>
+        <v>756</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="20" t="n">
+        <f aca="false">D23+D30</f>
+        <v>2293.5</v>
+      </c>
+      <c r="E31" s="19"/>
+      <c r="F31" s="20" t="n">
+        <f aca="false">F23+F30</f>
+        <v>3462</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A33:F33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2040,7 +2187,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -2053,7 +2200,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2061,7 +2208,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>74</v>
       </c>
@@ -2093,7 +2240,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -2103,55 +2250,55 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" s="14" t="n">
+        <v>109</v>
+      </c>
+      <c r="B5" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="C5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D5" s="16" t="n">
+      <c r="C5" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D5" s="14" t="n">
         <f aca="false">B5*C5</f>
         <v>300</v>
       </c>
-      <c r="E5" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F5" s="16" t="n">
+      <c r="E5" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F5" s="14" t="n">
         <f aca="false">B5*E5</f>
         <v>300</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B6" s="14" t="n">
+        <v>110</v>
+      </c>
+      <c r="B6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D6" s="16" t="n">
+      <c r="C6" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D6" s="14" t="n">
         <f aca="false">B6*C6</f>
         <v>200</v>
       </c>
-      <c r="E6" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F6" s="16" t="n">
+      <c r="E6" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F6" s="14" t="n">
         <f aca="false">B6*E6</f>
         <v>200</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -2163,22 +2310,22 @@
       <c r="A8" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D8" s="16" t="n">
+      <c r="C8" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D8" s="14" t="n">
         <f aca="false">B8*C8</f>
         <v>400</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="13" t="n">
         <f aca="false">Hypothèses!$B$5</f>
         <v>550</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="14" t="n">
         <f aca="false">B8*E8</f>
         <v>1100</v>
       </c>
@@ -2187,22 +2334,22 @@
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D9" s="16" t="n">
+      <c r="C9" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D9" s="14" t="n">
         <f aca="false">B9*C9</f>
         <v>400</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="13" t="n">
         <f aca="false">Hypothèses!$B$6</f>
         <v>500</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="14" t="n">
         <f aca="false">B9*E9</f>
         <v>1000</v>
       </c>
@@ -2211,46 +2358,46 @@
       <c r="A10" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="13" t="n">
         <f aca="false">Hypothèses!$B$9</f>
         <v>0</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="14" t="n">
         <f aca="false">B10*C10</f>
         <v>0</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="13" t="n">
         <f aca="false">Hypothèses!$B$11</f>
         <v>300</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="14" t="n">
         <f aca="false">B10*E10</f>
         <v>600</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B11" s="14" t="n">
+        <v>112</v>
+      </c>
+      <c r="B11" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="C11" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D11" s="16" t="n">
+      <c r="C11" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D11" s="14" t="n">
         <f aca="false">B11*C11</f>
         <v>100</v>
       </c>
-      <c r="E11" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F11" s="16" t="n">
+      <c r="E11" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F11" s="14" t="n">
         <f aca="false">B11*E11</f>
         <v>100</v>
       </c>
@@ -2267,72 +2414,72 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B13" s="14" t="n">
+        <v>113</v>
+      </c>
+      <c r="B13" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="C13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D13" s="16" t="n">
+      <c r="C13" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D13" s="14" t="n">
         <f aca="false">B13*C13</f>
         <v>300</v>
       </c>
-      <c r="E13" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F13" s="16" t="n">
+      <c r="E13" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F13" s="14" t="n">
         <f aca="false">B13*E13</f>
         <v>300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="14" t="n">
+        <v>114</v>
+      </c>
+      <c r="B14" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="C14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D14" s="16" t="n">
+      <c r="C14" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D14" s="14" t="n">
         <f aca="false">B14*C14</f>
         <v>1000</v>
       </c>
-      <c r="E14" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F14" s="16" t="n">
+      <c r="E14" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F14" s="14" t="n">
         <f aca="false">B14*E14</f>
         <v>1000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B15" s="14" t="n">
+        <v>115</v>
+      </c>
+      <c r="B15" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="C15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D15" s="16" t="n">
+      <c r="C15" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D15" s="14" t="n">
         <f aca="false">B15*C15</f>
         <v>300</v>
       </c>
-      <c r="E15" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F15" s="16" t="n">
+      <c r="E15" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F15" s="14" t="n">
         <f aca="false">B15*E15</f>
         <v>300</v>
       </c>
@@ -2341,22 +2488,22 @@
       <c r="A16" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B16" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D16" s="16" t="n">
+      <c r="C16" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D16" s="14" t="n">
         <f aca="false">B16*C16</f>
         <v>200</v>
       </c>
-      <c r="E16" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F16" s="16" t="n">
+      <c r="E16" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F16" s="14" t="n">
         <f aca="false">B16*E16</f>
         <v>200</v>
       </c>
@@ -2365,46 +2512,46 @@
       <c r="A17" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B17" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D17" s="16" t="n">
+      <c r="C17" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D17" s="14" t="n">
         <f aca="false">B17*C17</f>
         <v>200</v>
       </c>
-      <c r="E17" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F17" s="16" t="n">
+      <c r="E17" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F17" s="14" t="n">
         <f aca="false">B17*E17</f>
         <v>200</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18" s="14" t="n">
+        <v>116</v>
+      </c>
+      <c r="B18" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="C18" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D18" s="16" t="n">
+      <c r="C18" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D18" s="14" t="n">
         <f aca="false">B18*C18</f>
         <v>100</v>
       </c>
-      <c r="E18" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F18" s="16" t="n">
+      <c r="E18" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F18" s="14" t="n">
         <f aca="false">B18*E18</f>
         <v>100</v>
       </c>
@@ -2413,29 +2560,29 @@
       <c r="A19" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B19" s="14" t="n">
+      <c r="B19" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D19" s="16" t="n">
+      <c r="C19" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D19" s="14" t="n">
         <f aca="false">B19*C19</f>
         <v>200</v>
       </c>
-      <c r="E19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F19" s="16" t="n">
+      <c r="E19" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F19" s="14" t="n">
         <f aca="false">B19*E19</f>
         <v>200</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2445,24 +2592,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B21" s="14" t="n">
+        <v>118</v>
+      </c>
+      <c r="B21" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="C21" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="D21" s="16" t="n">
+      <c r="C21" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="D21" s="14" t="n">
         <f aca="false">B21*C21</f>
         <v>300</v>
       </c>
-      <c r="E21" s="15" t="n">
-        <f aca="false">Hypothèses!$B$8</f>
-        <v>200</v>
-      </c>
-      <c r="F21" s="16" t="n">
+      <c r="E21" s="13" t="n">
+        <f aca="false">Hypothèses!$B$8</f>
+        <v>200</v>
+      </c>
+      <c r="F21" s="14" t="n">
         <f aca="false">B21*E21</f>
         <v>300</v>
       </c>
@@ -2471,22 +2618,22 @@
       <c r="A22" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B22" s="14" t="n">
+      <c r="B22" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="15" t="n">
+      <c r="C22" s="13" t="n">
         <f aca="false">Hypothèses!$B$12</f>
         <v>50</v>
       </c>
-      <c r="D22" s="16" t="n">
+      <c r="D22" s="14" t="n">
         <f aca="false">B22*C22</f>
         <v>50</v>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="E22" s="13" t="n">
         <f aca="false">Hypothèses!$B$12</f>
         <v>50</v>
       </c>
-      <c r="F22" s="16" t="n">
+      <c r="F22" s="14" t="n">
         <f aca="false">B22*E22</f>
         <v>50</v>
       </c>
@@ -2497,12 +2644,12 @@
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
-      <c r="D23" s="17" t="n">
+      <c r="D23" s="15" t="n">
         <f aca="false">SUM(D5:D22)</f>
         <v>4050</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="17" t="n">
+      <c r="F23" s="15" t="n">
         <f aca="false">SUM(F5:F22)</f>
         <v>5950</v>
       </c>
@@ -2511,19 +2658,19 @@
       <c r="A24" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C24" s="18" t="n">
+      <c r="C24" s="16" t="n">
         <f aca="false">Hypothèses!$B$13</f>
         <v>0.15</v>
       </c>
-      <c r="D24" s="16" t="n">
+      <c r="D24" s="14" t="n">
         <f aca="false">D23*C24</f>
         <v>607.5</v>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="E24" s="16" t="n">
         <f aca="false">Hypothèses!$B$13</f>
         <v>0.15</v>
       </c>
-      <c r="F24" s="16" t="n">
+      <c r="F24" s="14" t="n">
         <f aca="false">F23*E24</f>
         <v>892.5</v>
       </c>
@@ -2532,19 +2679,19 @@
       <c r="A25" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="18" t="n">
+      <c r="C25" s="16" t="n">
         <f aca="false">Hypothèses!$B$14</f>
         <v>0.03</v>
       </c>
-      <c r="D25" s="16" t="n">
+      <c r="D25" s="14" t="n">
         <f aca="false">D23*C25</f>
         <v>121.5</v>
       </c>
-      <c r="E25" s="18" t="n">
+      <c r="E25" s="16" t="n">
         <f aca="false">Hypothèses!$B$14</f>
         <v>0.03</v>
       </c>
-      <c r="F25" s="16" t="n">
+      <c r="F25" s="14" t="n">
         <f aca="false">F23*E25</f>
         <v>178.5</v>
       </c>
@@ -2553,53 +2700,216 @@
       <c r="A26" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C26" s="18" t="n">
+      <c r="C26" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
-      <c r="D26" s="16" t="n">
+      <c r="D26" s="14" t="n">
         <f aca="false">D23*C26</f>
         <v>202.5</v>
       </c>
-      <c r="E26" s="18" t="n">
+      <c r="E26" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
         <v>0.05</v>
       </c>
-      <c r="F26" s="16" t="n">
+      <c r="F26" s="14" t="n">
         <f aca="false">F23*E26</f>
         <v>297.5</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="15" t="n">
         <f aca="false">D23+D24+D25+D26</f>
         <v>4981.5</v>
       </c>
       <c r="E27" s="3"/>
-      <c r="F27" s="17" t="n">
+      <c r="F27" s="15" t="n">
         <f aca="false">F23+F24+F25+F26</f>
         <v>7318.5</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B29" s="17" t="n">
+        <f aca="false">Hypothèses!$B$18</f>
+        <v>2</v>
+      </c>
+      <c r="C29" s="13" t="n">
+        <f aca="false">Hypothèses!$B$19</f>
+        <v>150</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <f aca="false">B29*C29</f>
+        <v>300</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <f aca="false">Hypothèses!$B$19</f>
+        <v>150</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <f aca="false">B29*E29</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B30" s="17" t="n">
+        <f aca="false">Hypothèses!$B$18*Hypothèses!$B$27</f>
+        <v>4</v>
+      </c>
+      <c r="C30" s="13" t="n">
+        <f aca="false">Hypothèses!$B$20</f>
+        <v>95</v>
+      </c>
+      <c r="D30" s="14" t="n">
+        <f aca="false">B30*C30</f>
+        <v>380</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <f aca="false">Hypothèses!$B$20</f>
+        <v>95</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <f aca="false">B30*E30</f>
+        <v>380</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B31" s="17" t="n">
+        <f aca="false">Hypothèses!$B$18*Hypothèses!$B$28</f>
+        <v>6</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <f aca="false">Hypothèses!$B$21</f>
+        <v>40</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <f aca="false">B31*C31</f>
+        <v>240</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <f aca="false">Hypothèses!$B$21</f>
+        <v>40</v>
+      </c>
+      <c r="F31" s="14" t="n">
+        <f aca="false">B31*E31</f>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" s="17" t="n">
+        <f aca="false">Hypothèses!$B$29</f>
+        <v>2</v>
+      </c>
+      <c r="C32" s="13" t="n">
+        <f aca="false">Hypothèses!$B$22</f>
+        <v>70</v>
+      </c>
+      <c r="D32" s="14" t="n">
+        <f aca="false">B32*C32</f>
+        <v>140</v>
+      </c>
+      <c r="E32" s="13" t="n">
+        <f aca="false">Hypothèses!$B$22</f>
+        <v>70</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <f aca="false">B32*E32</f>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="16" t="n">
+        <f aca="false">Hypothèses!$B$15</f>
+        <v>0.05</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <f aca="false">SUM(D29:D32)*C33</f>
+        <v>53</v>
+      </c>
+      <c r="E33" s="16" t="n">
+        <f aca="false">Hypothèses!$B$15</f>
+        <v>0.05</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <f aca="false">SUM(F29:F32)*E33</f>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="15" t="n">
+        <f aca="false">SUM(D29:D33)</f>
+        <v>1113</v>
+      </c>
+      <c r="E34" s="3"/>
+      <c r="F34" s="15" t="n">
+        <f aca="false">SUM(F29:F33)</f>
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="20" t="n">
+        <f aca="false">D27+D34</f>
+        <v>6094.5</v>
+      </c>
+      <c r="E35" s="19"/>
+      <c r="F35" s="20" t="n">
+        <f aca="false">F27+F34</f>
+        <v>8431.5</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A37:F37"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2616,148 +2926,336 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>115</v>
-      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="C3" s="21" t="n">
-        <f aca="false">Hypothèses!$B$18</f>
-        <v>2</v>
-      </c>
-      <c r="D3" s="16" t="n">
-        <f aca="false">C3*Hypothèses!$B$21</f>
-        <v>300</v>
+      <c r="A3" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>119</v>
-      </c>
-      <c r="C4" s="21" t="n">
-        <f aca="false">Hypothèses!$B$18*Hypothèses!$B$20</f>
-        <v>6</v>
-      </c>
-      <c r="D4" s="16" t="n">
-        <f aca="false">C4*Hypothèses!$B$22</f>
-        <v>570</v>
+        <v>125</v>
+      </c>
+      <c r="C4" s="13" t="n">
+        <f aca="false">'Format court'!$D$31</f>
+        <v>2293.5</v>
+      </c>
+      <c r="E4" s="13" t="n">
+        <f aca="false">'Format court'!$F$31</f>
+        <v>3462</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>121</v>
-      </c>
-      <c r="C5" s="21" t="n">
-        <f aca="false">Hypothèses!$B$18*(Hypothèses!$B$19+1)</f>
-        <v>8</v>
-      </c>
-      <c r="D5" s="16" t="n">
-        <f aca="false">C5*Hypothèses!$B$23</f>
-        <v>320</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" s="21" t="n">
-        <f aca="false">Hypothèses!$B$19</f>
-        <v>3</v>
-      </c>
-      <c r="D6" s="16" t="n">
-        <f aca="false">C6*Hypothèses!$B$24</f>
-        <v>210</v>
+        <v>126</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <f aca="false">'Format long'!$D$35</f>
+        <v>6094.5</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <f aca="false">'Format long'!$F$35</f>
+        <v>8431.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="17" t="n">
-        <f aca="false">SUM(D3:D6)</f>
-        <v>1400</v>
-      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="C8" s="18" t="n">
-        <f aca="false">Hypothèses!$B$15</f>
-        <v>0.05</v>
-      </c>
-      <c r="D8" s="16" t="n">
-        <f aca="false">D7*C8</f>
-        <v>70</v>
+      <c r="A8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="17" t="n">
-        <f aca="false">D7+D8</f>
-        <v>1470</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
-        <v>125</v>
-      </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
+      <c r="A9" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B9" s="17" t="n">
+        <f aca="false">Hypothèses!$B$31</f>
+        <v>4</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <f aca="false">B9*C4</f>
+        <v>9174</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <f aca="false">B9*E4</f>
+        <v>13848</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="17" t="n">
+        <f aca="false">Hypothèses!$B$32</f>
+        <v>2</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <f aca="false">B10*C5</f>
+        <v>12189</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <f aca="false">B10*E5</f>
+        <v>16863</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="15" t="n">
+        <f aca="false">SUM(D9:D10)</f>
+        <v>21363</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <f aca="false">SUM(E9:E10)</f>
+        <v>30711</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <f aca="false">B9*'Format court'!$D$30+B10*'Format long'!$D$34</f>
+        <v>5250</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <f aca="false">B9*'Format court'!$F$30+B10*'Format long'!$F$34</f>
+        <v>5250</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="23" t="n">
+        <f aca="false">B9+B10*4</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <f aca="false">D11*Hypothèses!$B$16</f>
+        <v>4272.6</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <f aca="false">E11*Hypothèses!$B$16</f>
+        <v>6142.2</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="D15" s="25" t="n">
+        <f aca="false">D11+D14</f>
+        <v>25635.6</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <f aca="false">E11+E14</f>
+        <v>36853.2</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <f aca="false">Hypothèses!$B$34</f>
+        <v>58000</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <f aca="false">Hypothèses!$B$34</f>
+        <v>58000</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D19" s="26" t="n">
+        <f aca="false">D11/D18</f>
+        <v>0.368327586206897</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <f aca="false">E11/E18</f>
+        <v>0.5295</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="D20" s="25" t="n">
+        <f aca="false">D18-D11</f>
+        <v>36637</v>
+      </c>
+      <c r="E20" s="25" t="n">
+        <f aca="false">E18-E11</f>
+        <v>27289</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D21" s="14" t="n">
+        <f aca="false">D11*Hypothèses!$B$35</f>
+        <v>27771.9</v>
+      </c>
+      <c r="E21" s="14" t="n">
+        <f aca="false">E11*Hypothèses!$B$35</f>
+        <v>39924.3</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <f aca="false">D18-D21</f>
+        <v>30228.1</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <f aca="false">E18-E21</f>
+        <v>18075.7</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <f aca="false">E11-D11</f>
+        <v>9348</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="E26" s="26" t="n">
+        <f aca="false">IF(D11=0,0,(E11-D11)/D11)</f>
+        <v>0.437578991714647</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21" t="s">
+        <v>146</v>
+      </c>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+    </row>
+    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A11:D11"/>
+  <mergeCells count="5">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A31:E31"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2774,544 +3272,101 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>2</v>
+        <v>151</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <f aca="false">'Format court'!$D$23+'Logistique vague'!$D$9*Hypothèses!$B$29</f>
-        <v>1659</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <f aca="false">'Format court'!$F$23+'Logistique vague'!$D$9*Hypothèses!$B$29</f>
-        <v>2243.25</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="C6" s="16" t="n">
-        <f aca="false">'Format long'!$D$27+'Logistique vague'!$D$9*Hypothèses!$B$30</f>
-        <v>5716.5</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <f aca="false">'Format long'!$F$27+'Logistique vague'!$D$9*Hypothèses!$B$30</f>
-        <v>8053.5</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="B10" s="21" t="n">
-        <f aca="false">Hypothèses!$B$27</f>
-        <v>4</v>
-      </c>
-      <c r="D10" s="16" t="n">
-        <f aca="false">B10*'Format court'!$D$23</f>
-        <v>5166</v>
-      </c>
-      <c r="E10" s="16" t="n">
-        <f aca="false">B10*'Format court'!$F$23</f>
-        <v>7503</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <f aca="false">Hypothèses!$B$28</f>
-        <v>2</v>
-      </c>
-      <c r="D11" s="16" t="n">
-        <f aca="false">B11*'Format long'!$D$27</f>
-        <v>9963</v>
-      </c>
-      <c r="E11" s="16" t="n">
-        <f aca="false">B11*'Format long'!$F$27</f>
-        <v>14637</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="B12" s="21" t="n">
-        <f aca="false">Hypothèses!$B$26</f>
-        <v>2</v>
-      </c>
-      <c r="D12" s="16" t="n">
-        <f aca="false">B12*'Logistique vague'!$D$9</f>
-        <v>2940</v>
-      </c>
-      <c r="E12" s="16" t="n">
-        <f aca="false">B12*'Logistique vague'!$D$9</f>
-        <v>2940</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="17" t="n">
-        <f aca="false">SUM(D10:D12)</f>
-        <v>18069</v>
-      </c>
-      <c r="E13" s="17" t="n">
-        <f aca="false">SUM(E10:E12)</f>
-        <v>25080</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="B14" s="22" t="n">
-        <f aca="false">B10+B11*4</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="16" t="n">
-        <f aca="false">D13*Hypothèses!$B$16</f>
-        <v>3613.8</v>
-      </c>
-      <c r="E15" s="16" t="n">
-        <f aca="false">E13*Hypothèses!$B$16</f>
-        <v>5016</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="D16" s="24" t="n">
-        <f aca="false">D13+D15</f>
-        <v>21682.8</v>
-      </c>
-      <c r="E16" s="24" t="n">
-        <f aca="false">E13+E15</f>
-        <v>30096</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="D19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$32</f>
-        <v>58000</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <f aca="false">Hypothèses!$B$32</f>
-        <v>58000</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D20" s="13" t="n">
-        <f aca="false">D13/D19</f>
-        <v>0.311534482758621</v>
-      </c>
-      <c r="E20" s="13" t="n">
-        <f aca="false">E13/E19</f>
-        <v>0.432413793103448</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="D21" s="24" t="n">
-        <f aca="false">D19-D13</f>
-        <v>39931</v>
-      </c>
-      <c r="E21" s="24" t="n">
-        <f aca="false">E19-E13</f>
-        <v>32920</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="D22" s="16" t="n">
-        <f aca="false">D13*Hypothèses!$B$33</f>
-        <v>23489.7</v>
-      </c>
-      <c r="E22" s="16" t="n">
-        <f aca="false">E13*Hypothèses!$B$33</f>
-        <v>32604</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="D23" s="17" t="n">
-        <f aca="false">D19-D22</f>
-        <v>34510.3</v>
-      </c>
-      <c r="E23" s="17" t="n">
-        <f aca="false">E19-E22</f>
-        <v>25396</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="E26" s="16" t="n">
-        <f aca="false">E13-D13</f>
-        <v>7011</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="E27" s="13" t="n">
-        <f aca="false">IF(D13=0,0,(E13-D13)/D13)</f>
-        <v>0.38801261829653</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-    </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-    </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="19" t="s">
+      <c r="C2" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A31:E31"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="17"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="C2" s="4" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="s">
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B5" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B6" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="C6" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="B5" s="5" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="D5" s="16" t="n">
-        <f aca="false">2*'Format court'!$D$23+'Format long'!$D$27+'Logistique vague'!$D$9</f>
-        <v>9034.5</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <f aca="false">2*'Format court'!$F$23+'Format long'!$F$27+'Logistique vague'!$D$9</f>
-        <v>12540</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
+      <c r="C7" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B6" s="5" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
+      <c r="B8" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>171</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="s">
-        <v>172</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="D8" s="16" t="n">
-        <f aca="false">2*'Format court'!$D$23+'Format long'!$D$27+'Logistique vague'!$D$9</f>
-        <v>9034.5</v>
-      </c>
-      <c r="E8" s="16" t="n">
-        <f aca="false">2*'Format court'!$F$23+'Format long'!$F$27+'Logistique vague'!$D$9</f>
-        <v>12540</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>175</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
-        <v>179</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="17" t="n">
-        <f aca="false">D5+D8</f>
-        <v>18069</v>
-      </c>
-      <c r="E12" s="17" t="n">
-        <f aca="false">E5+E8</f>
-        <v>25080</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="D13" s="16" t="n">
-        <f aca="false">D12-Synthèse!$D$13</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <f aca="false">E12-Synthèse!$E$13</f>
-        <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
AO ANFA : VTC à la place de la location de véhicule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoNCg8NnMhqnD1QgFW3cZV
</commit_message>
<xml_diff>
--- a/ao/anfa-2027/03_BUDGET.xlsx
+++ b/ao/anfa-2027/03_BUDGET.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="174">
   <si>
     <t xml:space="preserve">GRILLE DE COÛTS — AO ANFA 2027, Lot 1 vidéos métiers et formations (Pôle Audiovisuel L'Etudiant)</t>
   </si>
@@ -158,10 +158,13 @@
     <t xml:space="preserve">Barème URSSAF frais professionnels 2026 — base 2 repas/jour (référence CYRCE/BIOT2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Location véhicule sur place</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimation marché — utilitaire léger / citadine</t>
+    <t xml:space="preserve">Course VTC sur place (2 personnes + matériel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/course</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimation marché — course de 10 à 15 km en ville de province (gare, hôtel, site). Pas de location de véhicule (décision Martin, 28/10). À ajuster si le site est éloigné d'une gare</t>
   </si>
   <si>
     <t xml:space="preserve">LOGISTIQUE — PAR FORMAT (chaque vidéo est chiffrée seule, déplacement compris)</t>
@@ -185,10 +188,13 @@
     <t xml:space="preserve">Veille + jour de tournage</t>
   </si>
   <si>
-    <t xml:space="preserve">Format court : jours de véhicule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 journée de tournage</t>
+    <t xml:space="preserve">Format court : courses VTC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">courses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gare → hôtel la veille, hôtel → site, site → gare</t>
   </si>
   <si>
     <t xml:space="preserve">Format long : nuits sur place</t>
@@ -203,10 +209,10 @@
     <t xml:space="preserve">Veille + 2 jours de tournage</t>
   </si>
   <si>
-    <t xml:space="preserve">Format long : jours de véhicule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 journées de tournage</t>
+    <t xml:space="preserve">Format long : courses VTC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gare → hôtel, puis hôtel ↔ site sur 2 jours, site → gare</t>
   </si>
   <si>
     <t xml:space="preserve">VOLUMES</t>
@@ -332,7 +338,7 @@
     <t xml:space="preserve">Per diem repas (personnes × jours)</t>
   </si>
   <si>
-    <t xml:space="preserve">Location véhicule sur place (jours)</t>
+    <t xml:space="preserve">VTC sur place (courses)</t>
   </si>
   <si>
     <t xml:space="preserve">Provision imprévus (logistique)</t>
@@ -1333,23 +1339,23 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1357,91 +1363,91 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B25" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B26" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B27" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B28" s="10" t="n">
         <v>3</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B29" s="10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1449,35 +1455,35 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B31" s="10" t="n">
         <v>4</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B32" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1485,7 +1491,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B34" s="6" t="n">
         <v>58000</v>
@@ -1494,21 +1500,21 @@
         <v>21</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B35" s="11" t="n">
         <v>1.3</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1543,7 +1549,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1553,7 +1559,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1566,24 +1572,24 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1593,7 +1599,7 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>0.5</v>
@@ -1617,7 +1623,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1627,7 +1633,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>1</v>
@@ -1675,7 +1681,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>1</v>
@@ -1699,7 +1705,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>0.25</v>
@@ -1723,7 +1729,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -1733,7 +1739,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>1.5</v>
@@ -1757,7 +1763,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>0.5</v>
@@ -1781,7 +1787,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B14" s="12" t="n">
         <v>0.25</v>
@@ -1805,7 +1811,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B15" s="12" t="n">
         <v>0.25</v>
@@ -1829,7 +1835,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B16" s="12" t="n">
         <v>0.25</v>
@@ -1853,7 +1859,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B17" s="12" t="n">
         <v>0.5</v>
@@ -1877,7 +1883,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B18" s="12" t="n">
         <v>1</v>
@@ -1901,7 +1907,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1917,7 +1923,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C20" s="16" t="n">
         <f aca="false">Hypothèses!$B$13</f>
@@ -1959,7 +1965,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C22" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -1980,7 +1986,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1996,7 +2002,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -2006,7 +2012,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B25" s="17" t="n">
         <f aca="false">Hypothèses!$B$18</f>
@@ -2031,7 +2037,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B26" s="17" t="n">
         <f aca="false">Hypothèses!$B$18*Hypothèses!$B$24</f>
@@ -2056,7 +2062,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B27" s="17" t="n">
         <f aca="false">Hypothèses!$B$18*Hypothèses!$B$25</f>
@@ -2081,32 +2087,32 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B28" s="17" t="n">
         <f aca="false">Hypothèses!$B$26</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C28" s="13" t="n">
         <f aca="false">Hypothèses!$B$22</f>
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="D28" s="14" t="n">
         <f aca="false">B28*C28</f>
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E28" s="13" t="n">
         <f aca="false">Hypothèses!$B$22</f>
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="F28" s="14" t="n">
         <f aca="false">B28*E28</f>
-        <v>70</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C29" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -2114,7 +2120,7 @@
       </c>
       <c r="D29" s="14" t="n">
         <f aca="false">SUM(D25:D28)*C29</f>
-        <v>36</v>
+        <v>37.75</v>
       </c>
       <c r="E29" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -2122,44 +2128,44 @@
       </c>
       <c r="F29" s="14" t="n">
         <f aca="false">SUM(F25:F28)*E29</f>
-        <v>36</v>
+        <v>37.75</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D25:D29)</f>
-        <v>756</v>
+        <v>792.75</v>
       </c>
       <c r="E30" s="3"/>
       <c r="F30" s="15" t="n">
         <f aca="false">SUM(F25:F29)</f>
-        <v>756</v>
+        <v>792.75</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
       <c r="D31" s="20" t="n">
         <f aca="false">D23+D30</f>
-        <v>2293.5</v>
+        <v>2330.25</v>
       </c>
       <c r="E31" s="19"/>
       <c r="F31" s="20" t="n">
         <f aca="false">F23+F30</f>
-        <v>3462</v>
+        <v>3498.75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="21" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B33" s="21"/>
       <c r="C33" s="21"/>
@@ -2200,7 +2206,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2210,7 +2216,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2223,24 +2229,24 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -2250,7 +2256,7 @@
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>1.5</v>
@@ -2274,7 +2280,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1</v>
@@ -2298,7 +2304,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -2308,7 +2314,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>2</v>
@@ -2356,7 +2362,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>2</v>
@@ -2380,7 +2386,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>0.5</v>
@@ -2404,7 +2410,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -2414,7 +2420,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>1.5</v>
@@ -2438,7 +2444,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B14" s="12" t="n">
         <v>5</v>
@@ -2462,7 +2468,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B15" s="12" t="n">
         <v>1.5</v>
@@ -2486,7 +2492,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B16" s="12" t="n">
         <v>1</v>
@@ -2510,7 +2516,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B17" s="12" t="n">
         <v>1</v>
@@ -2534,7 +2540,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B18" s="12" t="n">
         <v>0.5</v>
@@ -2558,7 +2564,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B19" s="12" t="n">
         <v>1</v>
@@ -2582,7 +2588,7 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2592,7 +2598,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B21" s="12" t="n">
         <v>1.5</v>
@@ -2616,7 +2622,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B22" s="12" t="n">
         <v>1</v>
@@ -2640,7 +2646,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -2656,7 +2662,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C24" s="16" t="n">
         <f aca="false">Hypothèses!$B$13</f>
@@ -2698,7 +2704,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C26" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -2719,7 +2725,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2735,7 +2741,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -2745,7 +2751,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B29" s="17" t="n">
         <f aca="false">Hypothèses!$B$18</f>
@@ -2770,7 +2776,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B30" s="17" t="n">
         <f aca="false">Hypothèses!$B$18*Hypothèses!$B$27</f>
@@ -2795,7 +2801,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B31" s="17" t="n">
         <f aca="false">Hypothèses!$B$18*Hypothèses!$B$28</f>
@@ -2820,32 +2826,32 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B32" s="17" t="n">
         <f aca="false">Hypothèses!$B$29</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C32" s="13" t="n">
         <f aca="false">Hypothèses!$B$22</f>
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="D32" s="14" t="n">
         <f aca="false">B32*C32</f>
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="E32" s="13" t="n">
         <f aca="false">Hypothèses!$B$22</f>
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="F32" s="14" t="n">
         <f aca="false">B32*E32</f>
-        <v>140</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C33" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -2853,7 +2859,7 @@
       </c>
       <c r="D33" s="14" t="n">
         <f aca="false">SUM(D29:D32)*C33</f>
-        <v>53</v>
+        <v>54.75</v>
       </c>
       <c r="E33" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -2861,44 +2867,44 @@
       </c>
       <c r="F33" s="14" t="n">
         <f aca="false">SUM(F29:F32)*E33</f>
-        <v>53</v>
+        <v>54.75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="15" t="n">
         <f aca="false">SUM(D29:D33)</f>
-        <v>1113</v>
+        <v>1149.75</v>
       </c>
       <c r="E34" s="3"/>
       <c r="F34" s="15" t="n">
         <f aca="false">SUM(F29:F33)</f>
-        <v>1113</v>
+        <v>1149.75</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B35" s="19"/>
       <c r="C35" s="19"/>
       <c r="D35" s="20" t="n">
         <f aca="false">D27+D34</f>
-        <v>6094.5</v>
+        <v>6131.25</v>
       </c>
       <c r="E35" s="19"/>
       <c r="F35" s="20" t="n">
         <f aca="false">F27+F34</f>
-        <v>8431.5</v>
+        <v>8468.25</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B37" s="21"/>
       <c r="C37" s="21"/>
@@ -2936,7 +2942,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2945,7 +2951,7 @@
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2954,46 +2960,46 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C4" s="13" t="n">
         <f aca="false">'Format court'!$D$31</f>
-        <v>2293.5</v>
+        <v>2330.25</v>
       </c>
       <c r="E4" s="13" t="n">
         <f aca="false">'Format court'!$F$31</f>
-        <v>3462</v>
+        <v>3498.75</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C5" s="13" t="n">
         <f aca="false">'Format long'!$D$35</f>
-        <v>6094.5</v>
+        <v>6131.25</v>
       </c>
       <c r="E5" s="13" t="n">
         <f aca="false">'Format long'!$F$35</f>
-        <v>8431.5</v>
+        <v>8468.25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -3005,19 +3011,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">Hypothèses!$B$31</f>
@@ -3025,16 +3031,16 @@
       </c>
       <c r="D9" s="14" t="n">
         <f aca="false">B9*C4</f>
-        <v>9174</v>
+        <v>9321</v>
       </c>
       <c r="E9" s="14" t="n">
         <f aca="false">B9*E4</f>
-        <v>13848</v>
+        <v>13995</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">Hypothèses!$B$32</f>
@@ -3042,44 +3048,44 @@
       </c>
       <c r="D10" s="14" t="n">
         <f aca="false">B10*C5</f>
-        <v>12189</v>
+        <v>12262.5</v>
       </c>
       <c r="E10" s="14" t="n">
         <f aca="false">B10*E5</f>
-        <v>16863</v>
+        <v>16936.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="15" t="n">
         <f aca="false">SUM(D9:D10)</f>
-        <v>21363</v>
+        <v>21583.5</v>
       </c>
       <c r="E11" s="15" t="n">
         <f aca="false">SUM(E9:E10)</f>
-        <v>30711</v>
+        <v>30931.5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D12" s="14" t="n">
         <f aca="false">B9*'Format court'!$D$30+B10*'Format long'!$D$34</f>
-        <v>5250</v>
+        <v>5470.5</v>
       </c>
       <c r="E12" s="14" t="n">
         <f aca="false">B9*'Format court'!$F$30+B10*'Format long'!$F$34</f>
-        <v>5250</v>
+        <v>5470.5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B13" s="23" t="n">
         <f aca="false">B9+B10*4</f>
@@ -3092,29 +3098,29 @@
       </c>
       <c r="D14" s="14" t="n">
         <f aca="false">D11*Hypothèses!$B$16</f>
-        <v>4272.6</v>
+        <v>4316.7</v>
       </c>
       <c r="E14" s="14" t="n">
         <f aca="false">E11*Hypothèses!$B$16</f>
-        <v>6142.2</v>
+        <v>6186.3</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D15" s="25" t="n">
         <f aca="false">D11+D14</f>
-        <v>25635.6</v>
+        <v>25900.2</v>
       </c>
       <c r="E15" s="25" t="n">
         <f aca="false">E11+E14</f>
-        <v>36853.2</v>
+        <v>37117.8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -3123,7 +3129,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D18" s="13" t="n">
         <f aca="false">Hypothèses!$B$34</f>
@@ -3136,59 +3142,59 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D19" s="26" t="n">
         <f aca="false">D11/D18</f>
-        <v>0.368327586206897</v>
+        <v>0.372129310344828</v>
       </c>
       <c r="E19" s="26" t="n">
         <f aca="false">E11/E18</f>
-        <v>0.5295</v>
+        <v>0.533301724137931</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D20" s="25" t="n">
         <f aca="false">D18-D11</f>
-        <v>36637</v>
+        <v>36416.5</v>
       </c>
       <c r="E20" s="25" t="n">
         <f aca="false">E18-E11</f>
-        <v>27289</v>
+        <v>27068.5</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D21" s="14" t="n">
         <f aca="false">D11*Hypothèses!$B$35</f>
-        <v>27771.9</v>
+        <v>28058.55</v>
       </c>
       <c r="E21" s="14" t="n">
         <f aca="false">E11*Hypothèses!$B$35</f>
-        <v>39924.3</v>
+        <v>40210.95</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="24" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D22" s="15" t="n">
         <f aca="false">D18-D21</f>
-        <v>30228.1</v>
+        <v>29941.45</v>
       </c>
       <c r="E22" s="15" t="n">
         <f aca="false">E18-E21</f>
-        <v>18075.7</v>
+        <v>17789.05</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -3197,7 +3203,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E25" s="14" t="n">
         <f aca="false">E11-D11</f>
@@ -3206,16 +3212,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E26" s="26" t="n">
         <f aca="false">IF(D11=0,0,(E11-D11)/D11)</f>
-        <v>0.437578991714647</v>
+        <v>0.433108624643825</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="21"/>
@@ -3224,7 +3230,7 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B29" s="21"/>
       <c r="C29" s="21"/>
@@ -3233,7 +3239,7 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B30" s="21"/>
       <c r="C30" s="21"/>
@@ -3242,7 +3248,7 @@
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B31" s="21"/>
       <c r="C31" s="21"/>
@@ -3282,86 +3288,86 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="24" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AO ANFA : budget transmis aux OPS (30/10), version coûts ; points en suspens
</commit_message>
<xml_diff>
--- a/ao/anfa-2027/03_BUDGET.xlsx
+++ b/ao/anfa-2027/03_BUDGET.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="169">
   <si>
     <t xml:space="preserve">GRILLE DE COÛTS — AO ANFA 2027, Lot 1 vidéos métiers et formations (Pôle Audiovisuel L'Etudiant)</t>
   </si>
@@ -65,7 +65,7 @@
     <t xml:space="preserve">TAUX — SCÉNARIO A (base de l'offre : équipe interne de la cellule vidéo)</t>
   </si>
   <si>
-    <t xml:space="preserve">Taux interne (jour/personne, masse salariale)</t>
+    <t xml:space="preserve">Taux interne (jour/personne)</t>
   </si>
   <si>
     <t xml:space="preserve">Référentiel de Coûts Internes Pôle Audiovisuel — validé Direction</t>
@@ -242,15 +242,6 @@
     <t xml:space="preserve">RC / CDC §4 — accord-cadre sans minimum ; achats médias inclus (réponse ANFA du 28/10)</t>
   </si>
   <si>
-    <t xml:space="preserve">Repère marge plancher OPS (multiplicateur sur coût de revient)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BPU IDFM — Repères de marge (×1,3 plancher, ×1,5 standard secteur public). Décision OPS</t>
-  </si>
-  <si>
     <t xml:space="preserve">FORMAT COURT — vidéo métier ou formation, 60–120 s, verticale, immersive (4 par an minimum)</t>
   </si>
   <si>
@@ -347,7 +338,7 @@
     <t xml:space="preserve">Coût logistique (HT)</t>
   </si>
   <si>
-    <t xml:space="preserve">COÛT DE REVIENT COMPLET PAR VIDÉO (HT) — prix unitaire de bon de commande avant marge</t>
+    <t xml:space="preserve">COÛT COMPLET PAR VIDÉO (HT) — coût unitaire de bon de commande</t>
   </si>
   <si>
     <t xml:space="preserve">Chaque court est chiffré comme une commande autonome : 1 journée de tournage, déplacement et nuit sur place compris. Si deux vidéos sont commandées sur un même site, la logistique de l'une disparaît (le CDC autorise plusieurs vidéos par journée de tournage) : économie à répercuter ou non par les OPS.</t>
@@ -395,7 +386,7 @@
     <t xml:space="preserve">SYNTHÈSE — scénario annuel 2027, comparé au budget maximum du Lot 1</t>
   </si>
   <si>
-    <t xml:space="preserve">COÛT UNITAIRE COMPLET PAR VIDÉO (production + logistique) — base des prix unitaires des bons de commande</t>
+    <t xml:space="preserve">COÛT UNITAIRE COMPLET PAR VIDÉO (production + logistique) — base des coûts unitaires des bons de commande</t>
   </si>
   <si>
     <t xml:space="preserve">Format</t>
@@ -443,7 +434,7 @@
     <t xml:space="preserve">Coût de revient production annuel (TTC)</t>
   </si>
   <si>
-    <t xml:space="preserve">COMPARAISON AU BUDGET CLIENT (HT) — 58 k€ = production + diffusion + achats médias + marge</t>
+    <t xml:space="preserve">COMPARAISON AU BUDGET CLIENT (HT) — 58 k€ = production + diffusion + achats médias</t>
   </si>
   <si>
     <t xml:space="preserve">Budget annuel maximum Lot 1 (HT)</t>
@@ -452,13 +443,7 @@
     <t xml:space="preserve">Part du budget absorbée par la production (coût de revient)</t>
   </si>
   <si>
-    <t xml:space="preserve">Reste avant marge : médiatisation + marge OPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Production au prix plancher OPS (coût × repère de marge)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reste pour la médiatisation après marge plancher</t>
+    <t xml:space="preserve">Reste du budget pour la diffusion et les achats médias</t>
   </si>
   <si>
     <t xml:space="preserve">BASCULE A → B (si la cellule n'a pas la bande passante)</t>
@@ -470,13 +455,13 @@
     <t xml:space="preserve">Surcoût en % du scénario A</t>
   </si>
   <si>
-    <t xml:space="preserve">⚠️ Chiffrage prudent : chaque vidéo porte son propre déplacement. Si plusieurs commandes sont tournées sur un même site (autorisé par l'ANFA), la logistique partagée baisse le coût réel : marge de manœuvre pour les OPS.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠️ Le coût A est de la masse salariale déjà payée (taux 200 €/j), pas une dépense de trésorerie : il mesure la charge de la cellule, pas un achat. Matériel interne non valorisé (hors référentiel).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠️ La marge et la répartition médiatisation / marge relèvent des OPS. Le repère ×1,3 n'est affiché que pour visualiser ce qu'il reste à la diffusion ; ce n'est pas une décision.</t>
+    <t xml:space="preserve">⚠️ Chiffrage prudent : chaque vidéo porte son propre déplacement. Si plusieurs commandes sont tournées sur un même site (autorisé par l'ANFA), la logistique partagée baisse le coût réel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⚠️ Scénario A : taux interne du référentiel de coûts du pôle (200 €/j). Matériel interne non valorisé (hors référentiel).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⚠️ La répartition du budget entre production, médiatisation et achats médias relève des OPS.</t>
   </si>
   <si>
     <t xml:space="preserve">⚠️ Achats médias : la publicité ciblée vers les mineurs est très restreinte sur les grandes plateformes européennes ; la diffusion organique sur nos canaux reste l'atout principal (à chiffrer par les RS).</t>
@@ -552,13 +537,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;;\(#,##0&quot; €)&quot;;\-"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0"/>
-    <numFmt numFmtId="168" formatCode="0.0\x"/>
-    <numFmt numFmtId="169" formatCode="0.00"/>
+    <numFmt numFmtId="168" formatCode="0.00"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -716,7 +700,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -724,7 +712,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -736,11 +724,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -748,39 +736,35 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -788,11 +772,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -800,23 +784,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1075,448 +1059,435 @@
   <dimension ref="A1:D35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>550</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="6" t="n">
-        <v>200</v>
-      </c>
-      <c r="C8" s="7" t="s">
+      <c r="B8" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+    <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="10" t="n">
         <v>0.15</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="10" t="n">
         <v>0.03</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="10" t="n">
         <v>0.05</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B19" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="7" t="n">
         <v>95</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="6" t="n">
+      <c r="B21" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+    <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B22" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="10" t="n">
+      <c r="B24" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="10" t="n">
+      <c r="B25" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="10" t="n">
+      <c r="B26" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="9" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="9" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="10" t="n">
+      <c r="B28" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="10" t="n">
+      <c r="B29" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B31" s="10" t="n">
+      <c r="B31" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" s="9" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B34" s="6" t="n">
+      <c r="B34" s="7" t="n">
         <v>58000</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="D34" s="9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B35" s="11" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>74</v>
-      </c>
-    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
@@ -1539,67 +1510,67 @@
   <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="4" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>83</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>0.5</v>
@@ -1621,19 +1592,19 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>85</v>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>1</v>
@@ -1655,8 +1626,8 @@
         <v>550</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="12" t="n">
@@ -1679,9 +1650,9 @@
         <v>500</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>86</v>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>83</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>1</v>
@@ -1703,9 +1674,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>87</v>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>0.25</v>
@@ -1727,19 +1698,19 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>89</v>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>1.5</v>
@@ -1761,9 +1732,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>90</v>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>87</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>0.5</v>
@@ -1785,9 +1756,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>91</v>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="B14" s="12" t="n">
         <v>0.25</v>
@@ -1809,9 +1780,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>92</v>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="B15" s="12" t="n">
         <v>0.25</v>
@@ -1833,9 +1804,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>93</v>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>90</v>
       </c>
       <c r="B16" s="12" t="n">
         <v>0.25</v>
@@ -1857,9 +1828,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
-        <v>94</v>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="B17" s="12" t="n">
         <v>0.5</v>
@@ -1881,9 +1852,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>95</v>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>92</v>
       </c>
       <c r="B18" s="12" t="n">
         <v>1</v>
@@ -1905,25 +1876,25 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
       <c r="D19" s="15" t="n">
         <f aca="false">SUM(D5:D18)</f>
         <v>1250</v>
       </c>
-      <c r="E19" s="3"/>
+      <c r="E19" s="4"/>
       <c r="F19" s="15" t="n">
         <f aca="false">SUM(F5:F18)</f>
         <v>2200</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>97</v>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>94</v>
       </c>
       <c r="C20" s="16" t="n">
         <f aca="false">Hypothèses!$B$13</f>
@@ -1942,8 +1913,8 @@
         <v>330</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>26</v>
       </c>
       <c r="C21" s="16" t="n">
@@ -1963,9 +1934,9 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>98</v>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
+        <v>95</v>
       </c>
       <c r="C22" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -1984,35 +1955,35 @@
         <v>110</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
       <c r="D23" s="15" t="n">
         <f aca="false">D19+D20+D21+D22</f>
         <v>1537.5</v>
       </c>
-      <c r="E23" s="3"/>
+      <c r="E23" s="4"/>
       <c r="F23" s="15" t="n">
         <f aca="false">F19+F20+F21+F22</f>
         <v>2706</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>101</v>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
+        <v>98</v>
       </c>
       <c r="B25" s="17" t="n">
         <f aca="false">Hypothèses!$B$18</f>
@@ -2035,9 +2006,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>102</v>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="B26" s="17" t="n">
         <f aca="false">Hypothèses!$B$18*Hypothèses!$B$24</f>
@@ -2060,9 +2031,9 @@
         <v>190</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
-        <v>103</v>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>100</v>
       </c>
       <c r="B27" s="17" t="n">
         <f aca="false">Hypothèses!$B$18*Hypothèses!$B$25</f>
@@ -2085,9 +2056,9 @@
         <v>160</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>104</v>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
+        <v>101</v>
       </c>
       <c r="B28" s="17" t="n">
         <f aca="false">Hypothèses!$B$26</f>
@@ -2110,9 +2081,9 @@
         <v>105</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
-        <v>105</v>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>102</v>
       </c>
       <c r="C29" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -2131,25 +2102,25 @@
         <v>37.75</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D25:D29)</f>
         <v>792.75</v>
       </c>
-      <c r="E30" s="3"/>
+      <c r="E30" s="4"/>
       <c r="F30" s="15" t="n">
         <f aca="false">SUM(F25:F29)</f>
         <v>792.75</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
@@ -2165,7 +2136,7 @@
     </row>
     <row r="33" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="21" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B33" s="21"/>
       <c r="C33" s="21"/>
@@ -2196,67 +2167,67 @@
   <dimension ref="A1:F37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="A1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>111</v>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>108</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>1.5</v>
@@ -2278,9 +2249,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>112</v>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>109</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1</v>
@@ -2302,19 +2273,19 @@
         <v>200</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>85</v>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>2</v>
@@ -2336,8 +2307,8 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="12" t="n">
@@ -2360,9 +2331,9 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>86</v>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>83</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>2</v>
@@ -2384,9 +2355,9 @@
         <v>600</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>114</v>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>111</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>0.5</v>
@@ -2408,19 +2379,19 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>115</v>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>112</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>1.5</v>
@@ -2442,9 +2413,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>116</v>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>113</v>
       </c>
       <c r="B14" s="12" t="n">
         <v>5</v>
@@ -2466,9 +2437,9 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>117</v>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>114</v>
       </c>
       <c r="B15" s="12" t="n">
         <v>1.5</v>
@@ -2490,9 +2461,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>91</v>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="B16" s="12" t="n">
         <v>1</v>
@@ -2514,9 +2485,9 @@
         <v>200</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
-        <v>92</v>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="B17" s="12" t="n">
         <v>1</v>
@@ -2538,9 +2509,9 @@
         <v>200</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>118</v>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>115</v>
       </c>
       <c r="B18" s="12" t="n">
         <v>0.5</v>
@@ -2562,9 +2533,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>94</v>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="B19" s="12" t="n">
         <v>1</v>
@@ -2586,19 +2557,19 @@
         <v>200</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>120</v>
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="B21" s="12" t="n">
         <v>1.5</v>
@@ -2620,9 +2591,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>95</v>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>92</v>
       </c>
       <c r="B22" s="12" t="n">
         <v>1</v>
@@ -2644,25 +2615,25 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
       <c r="D23" s="15" t="n">
         <f aca="false">SUM(D5:D22)</f>
         <v>4050</v>
       </c>
-      <c r="E23" s="3"/>
+      <c r="E23" s="4"/>
       <c r="F23" s="15" t="n">
         <f aca="false">SUM(F5:F22)</f>
         <v>5950</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>97</v>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
+        <v>94</v>
       </c>
       <c r="C24" s="16" t="n">
         <f aca="false">Hypothèses!$B$13</f>
@@ -2681,8 +2652,8 @@
         <v>892.5</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
         <v>26</v>
       </c>
       <c r="C25" s="16" t="n">
@@ -2702,9 +2673,9 @@
         <v>178.5</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>98</v>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>95</v>
       </c>
       <c r="C26" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -2723,35 +2694,35 @@
         <v>297.5</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
       <c r="D27" s="15" t="n">
         <f aca="false">D23+D24+D25+D26</f>
         <v>4981.5</v>
       </c>
-      <c r="E27" s="3"/>
+      <c r="E27" s="4"/>
       <c r="F27" s="15" t="n">
         <f aca="false">F23+F24+F25+F26</f>
         <v>7318.5</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
-        <v>101</v>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>98</v>
       </c>
       <c r="B29" s="17" t="n">
         <f aca="false">Hypothèses!$B$18</f>
@@ -2774,9 +2745,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
-        <v>102</v>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="B30" s="17" t="n">
         <f aca="false">Hypothèses!$B$18*Hypothèses!$B$27</f>
@@ -2799,9 +2770,9 @@
         <v>380</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
-        <v>103</v>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
+        <v>100</v>
       </c>
       <c r="B31" s="17" t="n">
         <f aca="false">Hypothèses!$B$18*Hypothèses!$B$28</f>
@@ -2824,9 +2795,9 @@
         <v>240</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>104</v>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
+        <v>101</v>
       </c>
       <c r="B32" s="17" t="n">
         <f aca="false">Hypothèses!$B$29</f>
@@ -2849,9 +2820,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>105</v>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
+        <v>102</v>
       </c>
       <c r="C33" s="16" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -2870,25 +2841,25 @@
         <v>54.75</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
       <c r="D34" s="15" t="n">
         <f aca="false">SUM(D29:D33)</f>
         <v>1149.75</v>
       </c>
-      <c r="E34" s="3"/>
+      <c r="E34" s="4"/>
       <c r="F34" s="15" t="n">
         <f aca="false">SUM(F29:F33)</f>
         <v>1149.75</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B35" s="19"/>
       <c r="C35" s="19"/>
@@ -2904,7 +2875,7 @@
     </row>
     <row r="37" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B37" s="21"/>
       <c r="C37" s="21"/>
@@ -2935,45 +2906,45 @@
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>124</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>127</v>
       </c>
       <c r="C4" s="13" t="n">
         <f aca="false">'Format court'!$D$31</f>
@@ -2984,9 +2955,9 @@
         <v>3498.75</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>128</v>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>125</v>
       </c>
       <c r="C5" s="13" t="n">
         <f aca="false">'Format long'!$D$35</f>
@@ -2997,33 +2968,33 @@
         <v>8468.25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="4" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
         <v>130</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>133</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">Hypothèses!$B$31</f>
@@ -3038,9 +3009,9 @@
         <v>13995</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>134</v>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>131</v>
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">Hypothèses!$B$32</f>
@@ -3055,12 +3026,12 @@
         <v>16936.5</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
       <c r="D11" s="15" t="n">
         <f aca="false">SUM(D9:D10)</f>
         <v>21583.5</v>
@@ -3070,9 +3041,9 @@
         <v>30931.5</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D12" s="14" t="n">
         <f aca="false">B9*'Format court'!$D$30+B10*'Format long'!$D$34</f>
@@ -3083,17 +3054,17 @@
         <v>5470.5</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B13" s="23" t="n">
         <f aca="false">B9+B10*4</f>
         <v>12</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="14" t="n">
@@ -3105,9 +3076,9 @@
         <v>6186.3</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="24" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D15" s="25" t="n">
         <f aca="false">D11+D14</f>
@@ -3118,18 +3089,18 @@
         <v>37117.8</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>140</v>
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="D18" s="13" t="n">
         <f aca="false">Hypothèses!$B$34</f>
@@ -3140,9 +3111,9 @@
         <v>58000</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>141</v>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>138</v>
       </c>
       <c r="D19" s="26" t="n">
         <f aca="false">D11/D18</f>
@@ -3153,9 +3124,9 @@
         <v>0.533301724137931</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="24" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D20" s="25" t="n">
         <f aca="false">D18-D11</f>
@@ -3166,53 +3137,29 @@
         <v>27068.5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="D21" s="14" t="n">
-        <f aca="false">D11*Hypothèses!$B$35</f>
-        <v>28058.55</v>
-      </c>
-      <c r="E21" s="14" t="n">
-        <f aca="false">E11*Hypothèses!$B$35</f>
-        <v>40210.95</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="24" t="s">
-        <v>144</v>
-      </c>
-      <c r="D22" s="15" t="n">
-        <f aca="false">D18-D21</f>
-        <v>29941.45</v>
-      </c>
-      <c r="E22" s="15" t="n">
-        <f aca="false">E18-E21</f>
-        <v>17789.05</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>146</v>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
+        <v>141</v>
       </c>
       <c r="E25" s="14" t="n">
         <f aca="false">E11-D11</f>
         <v>9348</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>147</v>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="E26" s="26" t="n">
         <f aca="false">IF(D11=0,0,(E11-D11)/D11)</f>
@@ -3221,7 +3168,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="21"/>
@@ -3230,7 +3177,7 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B29" s="21"/>
       <c r="C29" s="21"/>
@@ -3239,7 +3186,7 @@
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B30" s="21"/>
       <c r="C30" s="21"/>
@@ -3248,7 +3195,7 @@
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B31" s="21"/>
       <c r="C31" s="21"/>
@@ -3281,93 +3228,93 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>155</v>
+      <c r="A1" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="24" t="s">
-        <v>156</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>158</v>
+        <v>151</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>161</v>
+        <v>154</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>164</v>
+        <v>157</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>165</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>167</v>
+        <v>160</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>168</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>170</v>
+        <v>163</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>171</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>